<commit_message>
feat(PDG-23): finalize DMW recruitment agencies mapping and normalization
</commit_message>
<xml_diff>
--- a/data/rules/mapping.xlsx
+++ b/data/rules/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D0E6D2-C1C4-4370-A313-49581D521CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F899D4-B510-48A0-830F-DDE2D11E34F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3791" uniqueCount="893">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3788" uniqueCount="891">
   <si>
     <t>Entity Category</t>
   </si>
@@ -2168,9 +2168,6 @@
     <t>"CFTC RED List record"</t>
   </si>
   <si>
-    <t>"Category:" | category</t>
-  </si>
-  <si>
     <t>Names associated with the organization</t>
   </si>
   <si>
@@ -2219,9 +2216,6 @@
     <t>"Listing Date"</t>
   </si>
   <si>
-    <t>"Data as Of"</t>
-  </si>
-  <si>
     <t>type.text | Organization Established Date | valueDate.isApproximate</t>
   </si>
   <si>
@@ -2294,9 +2288,6 @@
     <t>ENTITY_ADDRESS.NOTE</t>
   </si>
   <si>
-    <t>"Municipality/District: " | municipality_province</t>
-  </si>
-  <si>
     <t>Alternate or former names of the organization</t>
   </si>
   <si>
@@ -2417,9 +2408,6 @@
     <t>detail.web_address</t>
   </si>
   <si>
-    <t>expand(contact_number, /) * expand(eMail, /)</t>
-  </si>
-  <si>
     <t>Additional notes regarding the contact information</t>
   </si>
   <si>
@@ -2502,9 +2490,6 @@
   </si>
   <si>
     <t>Current status of the measure</t>
-  </si>
-  <si>
-    <t>license_status</t>
   </si>
   <si>
     <t>"License Status:" | license_status</t>
@@ -2831,9 +2816,6 @@
 offenses * saction_imposed * project * category</t>
   </si>
   <si>
-    <t xml:space="preserve">concat_path </t>
-  </si>
-  <si>
     <t>"Managed By" * "Contractor Of"</t>
   </si>
   <si>
@@ -2844,6 +2826,18 @@
   </si>
   <si>
     <t>"Sanction Imposed:" | saction_imposed</t>
+  </si>
+  <si>
+    <t>explode * explode</t>
+  </si>
+  <si>
+    <t>contact_number::/ * eMail::/</t>
+  </si>
+  <si>
+    <t>"Municipality/District:" | municipality_province</t>
+  </si>
+  <si>
+    <t>is_valid</t>
   </si>
 </sst>
 </file>
@@ -3061,7 +3055,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3139,6 +3133,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3510,16 +3507,16 @@
         <v>34</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="AN1" s="9"/>
       <c r="AO1" s="9"/>
@@ -12067,8 +12064,12 @@
       <c r="AK120" s="8" t="s">
         <v>650</v>
       </c>
-      <c r="AL120" s="8"/>
-      <c r="AM120" s="8"/>
+      <c r="AL120" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM120" s="9" t="s">
+        <v>680</v>
+      </c>
       <c r="AN120" s="9"/>
       <c r="AO120" s="9"/>
       <c r="AP120" s="9"/>
@@ -12825,12 +12826,8 @@
       </c>
       <c r="AJ128" s="8"/>
       <c r="AK128" s="8"/>
-      <c r="AL128" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="AM128" s="8" t="s">
-        <v>670</v>
-      </c>
+      <c r="AL128" s="5"/>
+      <c r="AM128" s="8"/>
       <c r="AN128" s="9"/>
       <c r="AO128" s="9"/>
       <c r="AP128" s="9"/>
@@ -12843,7 +12840,7 @@
         <v>146</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>85</v>
@@ -12921,7 +12918,7 @@
         <v>156</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>38</v>
@@ -13019,7 +13016,7 @@
         <v>167</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>38</v>
@@ -13051,7 +13048,7 @@
         <v>39</v>
       </c>
       <c r="O131" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="P131" s="5" t="s">
         <v>173</v>
@@ -13073,7 +13070,7 @@
         <v>177</v>
       </c>
       <c r="Y131" s="5" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="Z131" s="5" t="s">
         <v>39</v>
@@ -13095,19 +13092,19 @@
         <v>39</v>
       </c>
       <c r="AI131" s="8" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="AJ131" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AK131" s="8" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="AL131" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM131" s="8" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="AN131" s="9"/>
       <c r="AO131" s="9"/>
@@ -13411,7 +13408,7 @@
         <v>39</v>
       </c>
       <c r="G137" s="5" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H137" s="5" t="s">
         <v>213</v>
@@ -13549,13 +13546,13 @@
         <v>59</v>
       </c>
       <c r="I139" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="J139" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K139" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="L139" s="5"/>
       <c r="M139" s="5"/>
@@ -13595,16 +13592,10 @@
         <v>39</v>
       </c>
       <c r="AI139" s="8" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="AJ139" s="8"/>
       <c r="AK139" s="8"/>
-      <c r="AL139" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM139" s="9" t="s">
-        <v>681</v>
-      </c>
       <c r="AO139" s="9"/>
       <c r="AP139" s="9"/>
     </row>
@@ -13789,13 +13780,13 @@
         <v>59</v>
       </c>
       <c r="I143" s="6" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="J143" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K143" s="6" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="L143" s="5"/>
       <c r="M143" s="5"/>
@@ -13850,13 +13841,13 @@
         <v>59</v>
       </c>
       <c r="I144" s="6" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="J144" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K144" s="6" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="L144" s="5"/>
       <c r="M144" s="5"/>
@@ -13866,7 +13857,7 @@
         <v>55</v>
       </c>
       <c r="Q144" s="5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="R144" s="5" t="s">
         <v>55</v>
@@ -13886,7 +13877,7 @@
         <v>55</v>
       </c>
       <c r="AC144" s="5" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AD144" s="5"/>
       <c r="AE144" s="5"/>
@@ -13896,16 +13887,12 @@
         <v>55</v>
       </c>
       <c r="AI144" s="8" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="AJ144" s="5"/>
       <c r="AK144" s="5"/>
-      <c r="AL144" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="AM144" s="9" t="s">
-        <v>687</v>
-      </c>
+      <c r="AL144" s="5"/>
+      <c r="AM144" s="9"/>
       <c r="AO144" s="9"/>
       <c r="AP144" s="9"/>
     </row>
@@ -13931,13 +13918,13 @@
         <v>59</v>
       </c>
       <c r="I145" s="6" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="J145" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K145" s="6" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="L145" s="5"/>
       <c r="M145" s="5"/>
@@ -13965,7 +13952,7 @@
         <v>55</v>
       </c>
       <c r="AI145" s="8" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="AJ145" s="5"/>
       <c r="AK145" s="5"/>
@@ -14036,7 +14023,7 @@
         <v>323</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>85</v>
@@ -14098,7 +14085,7 @@
         <v>329</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>38</v>
@@ -14112,13 +14099,13 @@
         <v>59</v>
       </c>
       <c r="I148" s="6" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="J148" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K148" s="5" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="L148" s="5"/>
       <c r="M148" s="5"/>
@@ -14138,7 +14125,7 @@
         <v>55</v>
       </c>
       <c r="AA148" s="5" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="AB148" s="5"/>
       <c r="AC148" s="5"/>
@@ -14150,7 +14137,7 @@
         <v>55</v>
       </c>
       <c r="AI148" s="8" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="AJ148" s="5"/>
       <c r="AK148" s="5"/>
@@ -14240,13 +14227,13 @@
         <v>59</v>
       </c>
       <c r="I150" s="6" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="J150" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K150" s="5" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="L150" s="5"/>
       <c r="M150" s="5"/>
@@ -14274,7 +14261,7 @@
         <v>238</v>
       </c>
       <c r="AI150" s="19" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="AJ150" s="5"/>
       <c r="AK150" s="5"/>
@@ -14336,7 +14323,7 @@
         <v>39</v>
       </c>
       <c r="AI151" s="8" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="AJ151" s="8"/>
       <c r="AK151" s="8"/>
@@ -14354,7 +14341,7 @@
         <v>491</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>85</v>
@@ -14396,7 +14383,7 @@
         <v>149</v>
       </c>
       <c r="Y152" s="5" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Z152" s="5" t="s">
         <v>149</v>
@@ -14420,7 +14407,7 @@
       <c r="AO152" s="9"/>
       <c r="AP152" s="9"/>
     </row>
-    <row r="153" spans="1:42" ht="72.5">
+    <row r="153" spans="1:42" ht="58">
       <c r="A153" s="5" t="s">
         <v>644</v>
       </c>
@@ -14462,7 +14449,7 @@
         <v>213</v>
       </c>
       <c r="Q153" s="5" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="R153" s="5"/>
       <c r="S153" s="5"/>
@@ -14474,7 +14461,7 @@
         <v>213</v>
       </c>
       <c r="Y153" s="5" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="Z153" s="5" t="s">
         <v>213</v>
@@ -14498,13 +14485,13 @@
         <v>39</v>
       </c>
       <c r="AK153" s="8" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="AL153" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM153" s="8" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="AN153" s="9"/>
       <c r="AO153" s="9"/>
@@ -14754,7 +14741,7 @@
         <v>39</v>
       </c>
       <c r="Y157" s="5" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="Z157" s="5" t="s">
         <v>39</v>
@@ -14776,7 +14763,7 @@
         <v>39</v>
       </c>
       <c r="AM157" s="8" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="AN157" s="9"/>
       <c r="AO157" s="9"/>
@@ -14828,7 +14815,7 @@
         <v>39</v>
       </c>
       <c r="Y158" s="5" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="Z158" s="5" t="s">
         <v>39</v>
@@ -14902,7 +14889,7 @@
         <v>39</v>
       </c>
       <c r="Y159" s="5" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="Z159" s="5" t="s">
         <v>39</v>
@@ -14922,13 +14909,13 @@
         <v>55</v>
       </c>
       <c r="AK159" s="8" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="AL159" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM159" s="8" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="AN159" s="9"/>
       <c r="AO159" s="9"/>
@@ -14984,7 +14971,7 @@
         <v>39</v>
       </c>
       <c r="Y160" s="5" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="Z160" s="5" t="s">
         <v>39</v>
@@ -15046,7 +15033,7 @@
         <v>39</v>
       </c>
       <c r="Y161" s="5" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="Z161" s="5" t="s">
         <v>39</v>
@@ -15067,8 +15054,8 @@
       <c r="AL161" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="AM161" s="19" t="s">
-        <v>712</v>
+      <c r="AM161" s="27" t="s">
+        <v>889</v>
       </c>
       <c r="AN161" s="9"/>
       <c r="AO161" s="9"/>
@@ -15082,7 +15069,7 @@
         <v>420</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>85</v>
@@ -15128,7 +15115,7 @@
         <v>149</v>
       </c>
       <c r="Y162" s="5" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="Z162" s="5"/>
       <c r="AA162" s="5"/>
@@ -15280,7 +15267,7 @@
         <v>39</v>
       </c>
       <c r="Y164" s="5" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="Z164" s="5"/>
       <c r="AA164" s="5"/>
@@ -15514,7 +15501,7 @@
         <v>213</v>
       </c>
       <c r="Y168" s="5" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="Z168" s="5"/>
       <c r="AA168" s="5"/>
@@ -15974,7 +15961,7 @@
         <v>571</v>
       </c>
       <c r="Q174" s="5" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="R174" s="5"/>
       <c r="S174" s="5"/>
@@ -16040,7 +16027,7 @@
         <v>579</v>
       </c>
       <c r="Q175" s="5" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="R175" s="5"/>
       <c r="S175" s="5"/>
@@ -16062,19 +16049,19 @@
         <v>55</v>
       </c>
       <c r="AI175" s="8" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="AJ175" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AK175" s="8" t="s">
-        <v>889</v>
+        <v>883</v>
       </c>
       <c r="AL175" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM175" s="9" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AO175" s="9"/>
       <c r="AP175" s="9"/>
@@ -16178,7 +16165,7 @@
         <v>39</v>
       </c>
       <c r="Q177" s="5" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="R177" s="5"/>
       <c r="S177" s="5"/>
@@ -16200,19 +16187,19 @@
         <v>39</v>
       </c>
       <c r="AI177" s="8" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="AJ177" s="8" t="s">
         <v>180</v>
       </c>
       <c r="AK177" s="8" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="AL177" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM177" s="9" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="AO177" s="9"/>
       <c r="AP177" s="9"/>
@@ -16381,7 +16368,7 @@
         <v>55</v>
       </c>
       <c r="AI180" s="8" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="AJ180" s="8"/>
       <c r="AK180" s="8"/>
@@ -16399,7 +16386,7 @@
         <v>349</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>85</v>
@@ -16426,10 +16413,10 @@
       <c r="N181" s="5"/>
       <c r="O181" s="5"/>
       <c r="P181" s="5" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="Q181" s="5" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="R181" s="5"/>
       <c r="S181" s="5"/>
@@ -16465,7 +16452,7 @@
         <v>358</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>38</v>
@@ -16500,16 +16487,16 @@
         <v>364</v>
       </c>
       <c r="P182" s="5" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="Q182" s="5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="R182" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S182" s="5" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="T182" s="5"/>
       <c r="U182" s="5"/>
@@ -16519,7 +16506,7 @@
         <v>579</v>
       </c>
       <c r="Y182" s="5" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="Z182" s="5" t="s">
         <v>372</v>
@@ -16543,7 +16530,7 @@
         <v>55</v>
       </c>
       <c r="AK182" s="8" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="AL182" s="8"/>
       <c r="AM182" s="8"/>
@@ -16559,7 +16546,7 @@
         <v>375</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>38</v>
@@ -16594,10 +16581,10 @@
         <v>380</v>
       </c>
       <c r="P183" s="5" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="Q183" s="5" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="R183" s="5" t="s">
         <v>39</v>
@@ -16613,7 +16600,7 @@
         <v>180</v>
       </c>
       <c r="Y183" s="5" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="Z183" s="5" t="s">
         <v>379</v>
@@ -16637,7 +16624,7 @@
         <v>39</v>
       </c>
       <c r="AK183" s="8" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="AL183" s="8"/>
       <c r="AM183" s="8"/>
@@ -16775,7 +16762,7 @@
         <v>397</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>38</v>
@@ -16837,7 +16824,7 @@
         <v>391</v>
       </c>
       <c r="C187" s="5" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>38</v>
@@ -16929,13 +16916,13 @@
         <v>579</v>
       </c>
       <c r="Q188" s="5" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="R188" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S188" s="5" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="T188" s="5"/>
       <c r="U188" s="5"/>
@@ -16957,7 +16944,7 @@
         <v>55</v>
       </c>
       <c r="AK188" s="8" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="AL188" s="8"/>
       <c r="AM188" s="8"/>
@@ -16973,7 +16960,7 @@
         <v>415</v>
       </c>
       <c r="C189" s="5" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>85</v>
@@ -17003,7 +16990,7 @@
         <v>352</v>
       </c>
       <c r="Q189" s="5" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="R189" s="5"/>
       <c r="S189" s="5"/>
@@ -17039,7 +17026,7 @@
         <v>417</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>38</v>
@@ -17053,23 +17040,23 @@
         <v>59</v>
       </c>
       <c r="I190" s="6" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="J190" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K190" s="5" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="L190" s="5"/>
       <c r="M190" s="5"/>
       <c r="N190" s="5"/>
       <c r="O190" s="5"/>
       <c r="P190" s="5" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="Q190" s="5" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="R190" s="5"/>
       <c r="S190" s="5"/>
@@ -17091,15 +17078,15 @@
         <v>55</v>
       </c>
       <c r="AI190" s="8" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="AJ190" s="8"/>
       <c r="AK190" s="8"/>
-      <c r="AL190" s="19" t="s">
+      <c r="AL190" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="AM190" s="19" t="s">
-        <v>748</v>
+      <c r="AM190" s="27" t="s">
+        <v>745</v>
       </c>
       <c r="AN190" s="9"/>
       <c r="AO190" s="9"/>
@@ -17113,7 +17100,7 @@
         <v>418</v>
       </c>
       <c r="C191" s="5" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>38</v>
@@ -17127,13 +17114,13 @@
         <v>59</v>
       </c>
       <c r="I191" s="6" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="J191" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K191" s="5" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="L191" s="5"/>
       <c r="M191" s="5"/>
@@ -17143,7 +17130,7 @@
         <v>39</v>
       </c>
       <c r="Q191" s="5" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="R191" s="5"/>
       <c r="S191" s="5"/>
@@ -17165,13 +17152,15 @@
         <v>39</v>
       </c>
       <c r="AI191" s="8" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="AJ191" s="8"/>
       <c r="AK191" s="8"/>
-      <c r="AL191" s="19"/>
-      <c r="AM191" s="19" t="s">
-        <v>753</v>
+      <c r="AL191" s="26" t="s">
+        <v>887</v>
+      </c>
+      <c r="AM191" s="26" t="s">
+        <v>888</v>
       </c>
       <c r="AN191" s="9"/>
       <c r="AO191" s="9"/>
@@ -17185,7 +17174,7 @@
         <v>419</v>
       </c>
       <c r="C192" s="5" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>38</v>
@@ -17236,16 +17225,16 @@
         <v>644</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="C193" s="5" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>85</v>
       </c>
       <c r="E193" s="5" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="F193" s="5"/>
       <c r="G193" s="5"/>
@@ -17269,7 +17258,7 @@
         <v>149</v>
       </c>
       <c r="Q193" s="5" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="R193" s="5"/>
       <c r="S193" s="5"/>
@@ -17302,16 +17291,16 @@
         <v>644</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E194" s="5" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="F194" s="5"/>
       <c r="G194" s="5"/>
@@ -17319,13 +17308,13 @@
         <v>59</v>
       </c>
       <c r="I194" s="6" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="J194" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K194" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="L194" s="5"/>
       <c r="M194" s="5"/>
@@ -17335,7 +17324,7 @@
         <v>55</v>
       </c>
       <c r="Q194" s="5" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="R194" s="5" t="s">
         <v>39</v>
@@ -17374,16 +17363,16 @@
         <v>644</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="C195" s="5" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E195" s="5" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="F195" s="5" t="s">
         <v>140</v>
@@ -17395,13 +17384,13 @@
         <v>59</v>
       </c>
       <c r="I195" s="6" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="J195" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K195" s="5" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="L195" s="5"/>
       <c r="M195" s="5"/>
@@ -17431,7 +17420,7 @@
         <v>39</v>
       </c>
       <c r="AI195" s="8" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="AJ195" s="8"/>
       <c r="AK195" s="8"/>
@@ -17439,7 +17428,7 @@
         <v>39</v>
       </c>
       <c r="AM195" s="8" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="AN195" s="9"/>
       <c r="AO195" s="9"/>
@@ -17450,16 +17439,16 @@
         <v>644</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E196" s="5" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="F196" s="5"/>
       <c r="G196" s="5"/>
@@ -17477,7 +17466,7 @@
         <v>55</v>
       </c>
       <c r="S196" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="T196" s="5"/>
       <c r="U196" s="5"/>
@@ -17511,7 +17500,7 @@
         <v>599</v>
       </c>
       <c r="C197" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>85</v>
@@ -17629,19 +17618,19 @@
         <v>55</v>
       </c>
       <c r="AI198" s="8" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="AJ198" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AK198" s="8" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="AL198" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM198" s="8" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="AN198" s="9"/>
       <c r="AO198" s="9"/>
@@ -17707,19 +17696,19 @@
         <v>39</v>
       </c>
       <c r="AI199" s="8" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="AJ199" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AK199" s="8" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="AL199" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM199" s="8" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="AN199" s="9"/>
       <c r="AO199" s="9"/>
@@ -17775,13 +17764,13 @@
         <v>39</v>
       </c>
       <c r="AK200" s="8" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="AL200" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM200" s="8" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="AN200" s="9"/>
       <c r="AO200" s="9"/>
@@ -17795,7 +17784,7 @@
         <v>616</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>38</v>
@@ -17859,7 +17848,7 @@
         <v>39</v>
       </c>
       <c r="AM201" s="5" t="s">
-        <v>782</v>
+        <v>890</v>
       </c>
       <c r="AN201" s="9"/>
       <c r="AO201" s="9"/>
@@ -17927,13 +17916,13 @@
         <v>213</v>
       </c>
       <c r="AK202" s="8" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
       <c r="AL202" s="25" t="s">
-        <v>888</v>
+        <v>213</v>
       </c>
       <c r="AM202" s="8" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="AN202" s="9"/>
       <c r="AO202" s="9"/>
@@ -17947,7 +17936,7 @@
         <v>568</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>85</v>
@@ -18266,10 +18255,10 @@
       <c r="AH207" s="8"/>
       <c r="AI207" s="8"/>
       <c r="AJ207" s="26" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="AK207" s="26" t="s">
-        <v>890</v>
+        <v>884</v>
       </c>
       <c r="AL207" s="5"/>
       <c r="AM207" s="5"/>
@@ -18322,10 +18311,10 @@
       <c r="AH208" s="5"/>
       <c r="AI208" s="5"/>
       <c r="AJ208" s="26" t="s">
-        <v>891</v>
+        <v>885</v>
       </c>
       <c r="AK208" s="26" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="AL208" s="5"/>
       <c r="AM208" s="5"/>
@@ -18381,7 +18370,7 @@
         <v>149</v>
       </c>
       <c r="AI209" s="8" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="AJ209" s="8"/>
       <c r="AK209" s="8"/>
@@ -18439,7 +18428,7 @@
         <v>39</v>
       </c>
       <c r="AI210" s="5" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="AJ210" s="5"/>
       <c r="AK210" s="5"/>
@@ -18509,7 +18498,7 @@
     </row>
     <row r="212" spans="1:42" ht="14.5">
       <c r="A212" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B212" s="5" t="s">
         <v>36</v>
@@ -18551,7 +18540,7 @@
         <v>39</v>
       </c>
       <c r="U212" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="V212" s="5"/>
       <c r="W212" s="5"/>
@@ -18581,13 +18570,13 @@
     </row>
     <row r="213" spans="1:42" ht="14.5">
       <c r="A213" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B213" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="D213" s="5" t="s">
         <v>38</v>
@@ -18615,7 +18604,7 @@
         <v>55</v>
       </c>
       <c r="Q213" s="5" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="R213" s="5"/>
       <c r="S213" s="5"/>
@@ -18623,7 +18612,7 @@
         <v>55</v>
       </c>
       <c r="U213" s="5" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="V213" s="5"/>
       <c r="W213" s="5"/>
@@ -18635,7 +18624,7 @@
         <v>55</v>
       </c>
       <c r="AC213" s="7" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="AD213" s="5"/>
       <c r="AE213" s="5"/>
@@ -18653,13 +18642,13 @@
     </row>
     <row r="214" spans="1:42" ht="14.5">
       <c r="A214" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B214" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C214" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D214" s="5" t="s">
         <v>38</v>
@@ -18691,7 +18680,7 @@
         <v>39</v>
       </c>
       <c r="U214" s="5" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="V214" s="5"/>
       <c r="W214" s="5"/>
@@ -18721,7 +18710,7 @@
     </row>
     <row r="215" spans="1:42" ht="14.5">
       <c r="A215" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B215" s="5" t="s">
         <v>76</v>
@@ -18781,7 +18770,7 @@
     </row>
     <row r="216" spans="1:42" ht="14.5">
       <c r="A216" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B216" s="5" t="s">
         <v>83</v>
@@ -18835,7 +18824,7 @@
     </row>
     <row r="217" spans="1:42" ht="29">
       <c r="A217" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B217" s="5" t="s">
         <v>87</v>
@@ -18909,7 +18898,7 @@
     </row>
     <row r="218" spans="1:42" ht="29">
       <c r="A218" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B218" s="5" t="s">
         <v>90</v>
@@ -18999,7 +18988,7 @@
     </row>
     <row r="219" spans="1:42" ht="14.5">
       <c r="A219" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B219" s="5" t="s">
         <v>97</v>
@@ -19043,7 +19032,7 @@
         <v>55</v>
       </c>
       <c r="U219" s="5" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="V219" s="5"/>
       <c r="W219" s="5"/>
@@ -19081,7 +19070,7 @@
     </row>
     <row r="220" spans="1:42" ht="14.5">
       <c r="A220" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B220" s="5" t="s">
         <v>111</v>
@@ -19155,7 +19144,7 @@
     </row>
     <row r="221" spans="1:42" ht="58">
       <c r="A221" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B221" s="5" t="s">
         <v>122</v>
@@ -19199,7 +19188,7 @@
         <v>39</v>
       </c>
       <c r="U221" s="21" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="V221" s="5"/>
       <c r="W221" s="5"/>
@@ -19211,7 +19200,7 @@
         <v>55</v>
       </c>
       <c r="AC221" s="13" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="AD221" s="5"/>
       <c r="AE221" s="5"/>
@@ -19229,7 +19218,7 @@
     </row>
     <row r="222" spans="1:42" ht="14.5">
       <c r="A222" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B222" s="5" t="s">
         <v>136</v>
@@ -19273,7 +19262,7 @@
         <v>39</v>
       </c>
       <c r="U222" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="V222" s="5"/>
       <c r="W222" s="5"/>
@@ -19303,7 +19292,7 @@
     </row>
     <row r="223" spans="1:42" ht="14.5">
       <c r="A223" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B223" s="5" t="s">
         <v>138</v>
@@ -19369,13 +19358,13 @@
     </row>
     <row r="224" spans="1:42" ht="29">
       <c r="A224" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B224" s="5" t="s">
         <v>146</v>
       </c>
       <c r="C224" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>85</v>
@@ -19435,13 +19424,13 @@
     </row>
     <row r="225" spans="1:42" ht="43.5">
       <c r="A225" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B225" s="5" t="s">
         <v>156</v>
       </c>
       <c r="C225" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>38</v>
@@ -19509,13 +19498,13 @@
     </row>
     <row r="226" spans="1:42" ht="58">
       <c r="A226" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B226" s="5" t="s">
         <v>167</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D226" s="5" t="s">
         <v>38</v>
@@ -19553,7 +19542,7 @@
         <v>39</v>
       </c>
       <c r="U226" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="V226" s="5"/>
       <c r="W226" s="5"/>
@@ -19565,7 +19554,7 @@
         <v>39</v>
       </c>
       <c r="AC226" s="7" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="AD226" s="5"/>
       <c r="AE226" s="5"/>
@@ -19583,7 +19572,7 @@
     </row>
     <row r="227" spans="1:42" ht="14.5">
       <c r="A227" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B227" s="5" t="s">
         <v>200</v>
@@ -19635,7 +19624,7 @@
     </row>
     <row r="228" spans="1:42" ht="14.5">
       <c r="A228" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B228" s="5" t="s">
         <v>201</v>
@@ -19687,7 +19676,7 @@
     </row>
     <row r="229" spans="1:42" ht="14.5">
       <c r="A229" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B229" s="5" t="s">
         <v>202</v>
@@ -19739,7 +19728,7 @@
     </row>
     <row r="230" spans="1:42" ht="14.5">
       <c r="A230" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B230" s="5" t="s">
         <v>203</v>
@@ -19793,7 +19782,7 @@
     </row>
     <row r="231" spans="1:42" ht="14.5">
       <c r="A231" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B231" s="5" t="s">
         <v>209</v>
@@ -19849,7 +19838,7 @@
     </row>
     <row r="232" spans="1:42" ht="14.5">
       <c r="A232" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B232" s="5" t="s">
         <v>211</v>
@@ -19869,7 +19858,7 @@
         <v>59</v>
       </c>
       <c r="I232" s="6" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="J232" s="5"/>
       <c r="K232" s="5"/>
@@ -19907,13 +19896,13 @@
     </row>
     <row r="233" spans="1:42" ht="14.5">
       <c r="A233" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B233" s="5" t="s">
         <v>420</v>
       </c>
       <c r="C233" s="5" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>85</v>
@@ -19973,7 +19962,7 @@
     </row>
     <row r="234" spans="1:42" ht="43.5">
       <c r="A234" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B234" s="5" t="s">
         <v>425</v>
@@ -20043,7 +20032,7 @@
     </row>
     <row r="235" spans="1:42" ht="43.5">
       <c r="A235" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B235" s="5" t="s">
         <v>430</v>
@@ -20113,7 +20102,7 @@
     </row>
     <row r="236" spans="1:42" ht="14.5">
       <c r="A236" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B236" s="5" t="s">
         <v>437</v>
@@ -20165,7 +20154,7 @@
     </row>
     <row r="237" spans="1:42" ht="14.5">
       <c r="A237" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B237" s="5" t="s">
         <v>438</v>
@@ -20217,7 +20206,7 @@
     </row>
     <row r="238" spans="1:42" ht="14.5">
       <c r="A238" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B238" s="5" t="s">
         <v>439</v>
@@ -20269,7 +20258,7 @@
     </row>
     <row r="239" spans="1:42" ht="43.5">
       <c r="A239" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B239" s="5" t="s">
         <v>440</v>
@@ -20293,7 +20282,7 @@
         <v>59</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="J239" s="5"/>
       <c r="K239" s="5"/>
@@ -20335,13 +20324,13 @@
     </row>
     <row r="240" spans="1:42" ht="29">
       <c r="A240" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B240" s="5" t="s">
         <v>349</v>
       </c>
       <c r="C240" s="5" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>85</v>
@@ -20364,10 +20353,10 @@
       <c r="N240" s="5"/>
       <c r="O240" s="5"/>
       <c r="P240" s="5" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="Q240" s="5" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="R240" s="5"/>
       <c r="S240" s="5"/>
@@ -20397,13 +20386,13 @@
     </row>
     <row r="241" spans="1:42" ht="188.5">
       <c r="A241" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B241" s="5" t="s">
         <v>358</v>
       </c>
       <c r="C241" s="5" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>38</v>
@@ -20415,7 +20404,7 @@
         <v>372</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="H241" s="5" t="s">
         <v>361</v>
@@ -20430,10 +20419,10 @@
       <c r="N241" s="5"/>
       <c r="O241" s="5"/>
       <c r="P241" s="5" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="Q241" s="5" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="R241" s="5"/>
       <c r="S241" s="5"/>
@@ -20441,7 +20430,7 @@
         <v>55</v>
       </c>
       <c r="U241" s="5" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="V241" s="5"/>
       <c r="W241" s="5"/>
@@ -20453,7 +20442,7 @@
         <v>93</v>
       </c>
       <c r="AC241" s="7" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="AD241" s="5"/>
       <c r="AE241" s="5"/>
@@ -20471,13 +20460,13 @@
     </row>
     <row r="242" spans="1:42" ht="145">
       <c r="A242" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B242" s="5" t="s">
         <v>375</v>
       </c>
       <c r="C242" s="5" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="D242" s="5" t="s">
         <v>38</v>
@@ -20489,13 +20478,13 @@
         <v>379</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="H242" s="5" t="s">
         <v>377</v>
       </c>
       <c r="I242" s="6" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="J242" s="5"/>
       <c r="K242" s="5"/>
@@ -20504,10 +20493,10 @@
       <c r="N242" s="5"/>
       <c r="O242" s="5"/>
       <c r="P242" s="5" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="Q242" s="5" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="R242" s="5"/>
       <c r="S242" s="5"/>
@@ -20515,7 +20504,7 @@
         <v>39</v>
       </c>
       <c r="U242" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="V242" s="5"/>
       <c r="W242" s="5"/>
@@ -20527,7 +20516,7 @@
         <v>180</v>
       </c>
       <c r="AC242" s="7" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="AD242" s="5"/>
       <c r="AE242" s="5"/>
@@ -20545,7 +20534,7 @@
     </row>
     <row r="243" spans="1:42" ht="29">
       <c r="A243" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B243" s="5" t="s">
         <v>390</v>
@@ -20597,13 +20586,13 @@
     </row>
     <row r="244" spans="1:42" ht="14.5">
       <c r="A244" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B244" s="5" t="s">
         <v>397</v>
       </c>
       <c r="C244" s="5" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>38</v>
@@ -20655,13 +20644,13 @@
     </row>
     <row r="245" spans="1:42" ht="14.5">
       <c r="A245" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B245" s="5" t="s">
         <v>391</v>
       </c>
       <c r="C245" s="5" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>38</v>
@@ -20713,13 +20702,13 @@
     </row>
     <row r="246" spans="1:42" ht="14.5">
       <c r="A246" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B246" s="5" t="s">
         <v>401</v>
       </c>
       <c r="C246" s="5" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>38</v>
@@ -20771,7 +20760,7 @@
     </row>
     <row r="247" spans="1:42" ht="174">
       <c r="A247" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B247" s="5" t="s">
         <v>406</v>
@@ -20800,10 +20789,10 @@
       <c r="N247" s="5"/>
       <c r="O247" s="5"/>
       <c r="P247" s="5" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="Q247" s="5" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="R247" s="5"/>
       <c r="S247" s="5"/>
@@ -20833,7 +20822,7 @@
     </row>
     <row r="248" spans="1:42" ht="14.5">
       <c r="A248" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B248" s="5" t="s">
         <v>258</v>
@@ -20867,7 +20856,7 @@
         <v>149</v>
       </c>
       <c r="Q248" s="5" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="R248" s="5"/>
       <c r="S248" s="5"/>
@@ -20897,7 +20886,7 @@
     </row>
     <row r="249" spans="1:42" ht="29">
       <c r="A249" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B249" s="5" t="s">
         <v>264</v>
@@ -20917,7 +20906,7 @@
         <v>59</v>
       </c>
       <c r="I249" s="6" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
       <c r="J249" s="5"/>
       <c r="K249" s="5"/>
@@ -20929,7 +20918,7 @@
         <v>39</v>
       </c>
       <c r="Q249" s="5" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="R249" s="5"/>
       <c r="S249" s="5"/>
@@ -20959,7 +20948,7 @@
     </row>
     <row r="250" spans="1:42" ht="14.5">
       <c r="A250" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B250" s="5" t="s">
         <v>276</v>
@@ -21013,7 +21002,7 @@
     </row>
     <row r="251" spans="1:42" ht="14.5">
       <c r="A251" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B251" s="5" t="s">
         <v>278</v>
@@ -21067,7 +21056,7 @@
     </row>
     <row r="252" spans="1:42" ht="14.5">
       <c r="A252" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B252" s="5" t="s">
         <v>280</v>
@@ -21121,7 +21110,7 @@
     </row>
     <row r="253" spans="1:42" ht="14.5">
       <c r="A253" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B253" s="5" t="s">
         <v>282</v>
@@ -21141,7 +21130,7 @@
         <v>59</v>
       </c>
       <c r="I253" s="6" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="J253" s="5"/>
       <c r="K253" s="5"/>
@@ -21179,7 +21168,7 @@
     </row>
     <row r="254" spans="1:42" ht="29">
       <c r="A254" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B254" s="5" t="s">
         <v>285</v>
@@ -21199,7 +21188,7 @@
         <v>59</v>
       </c>
       <c r="I254" s="6" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="J254" s="5"/>
       <c r="K254" s="5"/>
@@ -21211,7 +21200,7 @@
         <v>55</v>
       </c>
       <c r="Q254" s="5" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="R254" s="5"/>
       <c r="S254" s="5"/>
@@ -21241,7 +21230,7 @@
     </row>
     <row r="255" spans="1:42" ht="14.5">
       <c r="A255" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B255" s="5" t="s">
         <v>293</v>
@@ -21295,7 +21284,7 @@
     </row>
     <row r="256" spans="1:42" ht="14.5">
       <c r="A256" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B256" s="5" t="s">
         <v>286</v>
@@ -21349,13 +21338,13 @@
     </row>
     <row r="257" spans="1:42" ht="29">
       <c r="A257" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B257" s="5" t="s">
         <v>323</v>
       </c>
       <c r="C257" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>85</v>
@@ -21377,7 +21366,7 @@
         <v>149</v>
       </c>
       <c r="Q257" s="5" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="R257" s="5"/>
       <c r="S257" s="5"/>
@@ -21407,13 +21396,13 @@
     </row>
     <row r="258" spans="1:42" ht="14.5">
       <c r="A258" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B258" s="5" t="s">
         <v>329</v>
       </c>
       <c r="C258" s="5" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>38</v>
@@ -21435,7 +21424,7 @@
         <v>55</v>
       </c>
       <c r="Q258" s="5" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="R258" s="5"/>
       <c r="S258" s="5"/>
@@ -21465,7 +21454,7 @@
     </row>
     <row r="259" spans="1:42" ht="14.5">
       <c r="A259" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B259" s="5" t="s">
         <v>335</v>
@@ -21519,7 +21508,7 @@
     </row>
     <row r="260" spans="1:42" ht="29">
       <c r="A260" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B260" s="5" t="s">
         <v>337</v>
@@ -21547,7 +21536,7 @@
         <v>39</v>
       </c>
       <c r="Q260" s="5" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="R260" s="5"/>
       <c r="S260" s="5"/>
@@ -21577,7 +21566,7 @@
     </row>
     <row r="261" spans="1:42" ht="14.5">
       <c r="A261" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B261" s="5" t="s">
         <v>345</v>
@@ -21631,13 +21620,13 @@
     </row>
     <row r="262" spans="1:42" ht="14.5">
       <c r="A262" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B262" s="5" t="s">
         <v>491</v>
       </c>
       <c r="C262" s="5" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>85</v>
@@ -21689,7 +21678,7 @@
     </row>
     <row r="263" spans="1:42" ht="14.5">
       <c r="A263" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B263" s="5" t="s">
         <v>498</v>
@@ -21751,7 +21740,7 @@
     </row>
     <row r="264" spans="1:42" ht="29">
       <c r="A264" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B264" s="5" t="s">
         <v>507</v>
@@ -21809,7 +21798,7 @@
     </row>
     <row r="265" spans="1:42" ht="29">
       <c r="A265" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B265" s="5" t="s">
         <v>511</v>
@@ -21867,7 +21856,7 @@
     </row>
     <row r="266" spans="1:42" ht="29">
       <c r="A266" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B266" s="5" t="s">
         <v>515</v>
@@ -21925,7 +21914,7 @@
     </row>
     <row r="267" spans="1:42" ht="29">
       <c r="A267" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B267" s="5" t="s">
         <v>519</v>
@@ -21983,7 +21972,7 @@
     </row>
     <row r="268" spans="1:42" ht="29">
       <c r="A268" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B268" s="5" t="s">
         <v>530</v>
@@ -22041,7 +22030,7 @@
     </row>
     <row r="269" spans="1:42" ht="14.5">
       <c r="A269" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B269" s="5" t="s">
         <v>524</v>
@@ -22099,7 +22088,7 @@
     </row>
     <row r="270" spans="1:42" ht="29">
       <c r="A270" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B270" s="5" t="s">
         <v>535</v>
@@ -22157,7 +22146,7 @@
     </row>
     <row r="271" spans="1:42" ht="14.5">
       <c r="A271" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B271" s="5" t="s">
         <v>541</v>
@@ -22211,19 +22200,19 @@
     </row>
     <row r="272" spans="1:42" ht="14.5">
       <c r="A272" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="C272" s="5" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="D272" s="5" t="s">
         <v>85</v>
       </c>
       <c r="E272" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F272" s="5"/>
       <c r="G272" s="5"/>
@@ -22243,7 +22232,7 @@
         <v>149</v>
       </c>
       <c r="Q272" s="5" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="R272" s="5"/>
       <c r="S272" s="5"/>
@@ -22273,19 +22262,19 @@
     </row>
     <row r="273" spans="1:42" ht="14.5">
       <c r="A273" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>836</v>
+        <v>831</v>
       </c>
       <c r="C273" s="5" t="s">
-        <v>837</v>
+        <v>832</v>
       </c>
       <c r="D273" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E273" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F273" s="5"/>
       <c r="G273" s="5"/>
@@ -22293,7 +22282,7 @@
         <v>59</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="J273" s="5"/>
       <c r="K273" s="5"/>
@@ -22305,7 +22294,7 @@
         <v>39</v>
       </c>
       <c r="Q273" s="5" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="R273" s="5"/>
       <c r="S273" s="5"/>
@@ -22335,19 +22324,19 @@
     </row>
     <row r="274" spans="1:42" ht="14.5">
       <c r="A274" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="C274" s="5" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="D274" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E274" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F274" s="5"/>
       <c r="G274" s="5"/>
@@ -22355,7 +22344,7 @@
         <v>59</v>
       </c>
       <c r="I274" s="6" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="J274" s="5"/>
       <c r="K274" s="5"/>
@@ -22367,7 +22356,7 @@
         <v>39</v>
       </c>
       <c r="Q274" s="5" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="R274" s="5"/>
       <c r="S274" s="5"/>
@@ -22397,19 +22386,19 @@
     </row>
     <row r="275" spans="1:42" ht="14.5">
       <c r="A275" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="C275" s="5" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="D275" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E275" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F275" s="5"/>
       <c r="G275" s="5"/>
@@ -22417,7 +22406,7 @@
         <v>59</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="J275" s="5"/>
       <c r="K275" s="5"/>
@@ -22429,7 +22418,7 @@
         <v>39</v>
       </c>
       <c r="Q275" s="5" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="R275" s="5"/>
       <c r="S275" s="5"/>
@@ -22459,19 +22448,19 @@
     </row>
     <row r="276" spans="1:42" ht="29">
       <c r="A276" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="C276" s="5" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E276" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F276" s="5"/>
       <c r="G276" s="5"/>
@@ -22513,19 +22502,19 @@
     </row>
     <row r="277" spans="1:42" ht="14.5">
       <c r="A277" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="C277" s="5" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="D277" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E277" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F277" s="5"/>
       <c r="G277" s="5"/>
@@ -22533,7 +22522,7 @@
         <v>59</v>
       </c>
       <c r="I277" s="6" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="J277" s="5"/>
       <c r="K277" s="5"/>
@@ -22545,7 +22534,7 @@
         <v>39</v>
       </c>
       <c r="Q277" s="5" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="R277" s="5"/>
       <c r="S277" s="5"/>
@@ -22575,19 +22564,19 @@
     </row>
     <row r="278" spans="1:42" ht="14.5">
       <c r="A278" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="C278" s="5" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="D278" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E278" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F278" s="5"/>
       <c r="G278" s="5"/>
@@ -22603,7 +22592,7 @@
         <v>39</v>
       </c>
       <c r="Q278" s="5" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="R278" s="5"/>
       <c r="S278" s="5"/>
@@ -22633,17 +22622,17 @@
     </row>
     <row r="279" spans="1:42" ht="14.5">
       <c r="A279" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="C279" s="5"/>
       <c r="D279" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E279" s="5" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="F279" s="5"/>
       <c r="G279" s="5"/>
@@ -22651,7 +22640,7 @@
         <v>59</v>
       </c>
       <c r="I279" s="6" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="J279" s="5"/>
       <c r="K279" s="5"/>
@@ -22663,7 +22652,7 @@
         <v>39</v>
       </c>
       <c r="Q279" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="R279" s="5"/>
       <c r="S279" s="5"/>
@@ -22693,17 +22682,17 @@
     </row>
     <row r="280" spans="1:42" ht="14.5">
       <c r="A280" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="C280" s="5"/>
       <c r="D280" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E280" s="5" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="F280" s="5"/>
       <c r="G280" s="5"/>
@@ -22711,7 +22700,7 @@
         <v>59</v>
       </c>
       <c r="I280" s="6" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="J280" s="5"/>
       <c r="K280" s="5"/>
@@ -22749,31 +22738,31 @@
     </row>
     <row r="281" spans="1:42" ht="14.5">
       <c r="A281" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="C281" s="5" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="D281" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E281" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F281" s="5" t="s">
         <v>39</v>
       </c>
       <c r="G281" s="5" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="H281" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I281" s="6" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="J281" s="5"/>
       <c r="K281" s="5"/>
@@ -22811,19 +22800,19 @@
     </row>
     <row r="282" spans="1:42" ht="14.5">
       <c r="A282" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B282" s="5" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="C282" s="5" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E282" s="5" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="F282" s="5" t="s">
         <v>39</v>
@@ -22869,17 +22858,17 @@
     </row>
     <row r="283" spans="1:42" ht="14.5">
       <c r="A283" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="C283" s="5"/>
       <c r="D283" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E283" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="F283" s="5"/>
       <c r="G283" s="5"/>
@@ -22897,7 +22886,7 @@
       <c r="O283" s="5"/>
       <c r="P283" s="5"/>
       <c r="Q283" s="5" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="R283" s="5"/>
       <c r="S283" s="5"/>
@@ -22927,17 +22916,17 @@
     </row>
     <row r="284" spans="1:42" ht="43.5">
       <c r="A284" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B284" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C284" s="5"/>
       <c r="D284" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E284" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="F284" s="5"/>
       <c r="G284" s="5"/>
@@ -22945,7 +22934,7 @@
         <v>59</v>
       </c>
       <c r="I284" s="6" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="J284" s="5"/>
       <c r="K284" s="5"/>
@@ -22957,7 +22946,7 @@
         <v>579</v>
       </c>
       <c r="Q284" s="5" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="R284" s="5"/>
       <c r="S284" s="5"/>
@@ -22987,17 +22976,17 @@
     </row>
     <row r="285" spans="1:42" ht="43.5">
       <c r="A285" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B285" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="C285" s="5"/>
       <c r="D285" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E285" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="F285" s="5"/>
       <c r="G285" s="5"/>
@@ -23005,7 +22994,7 @@
         <v>59</v>
       </c>
       <c r="I285" s="6" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="J285" s="5"/>
       <c r="K285" s="5"/>
@@ -23017,7 +23006,7 @@
         <v>594</v>
       </c>
       <c r="Q285" s="5" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="R285" s="5"/>
       <c r="S285" s="5"/>
@@ -23047,7 +23036,7 @@
     </row>
     <row r="286" spans="1:42" ht="14.5">
       <c r="A286" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B286" s="5" t="s">
         <v>445</v>
@@ -23109,7 +23098,7 @@
     </row>
     <row r="287" spans="1:42" ht="14.5">
       <c r="A287" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B287" s="5" t="s">
         <v>450</v>
@@ -23179,7 +23168,7 @@
     </row>
     <row r="288" spans="1:42" ht="14.5">
       <c r="A288" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B288" s="5" t="s">
         <v>453</v>
@@ -23249,7 +23238,7 @@
     </row>
     <row r="289" spans="1:42" ht="29">
       <c r="A289" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B289" s="5" t="s">
         <v>463</v>
@@ -23319,7 +23308,7 @@
     </row>
     <row r="290" spans="1:42" ht="14.5">
       <c r="A290" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B290" s="5" t="s">
         <v>472</v>
@@ -23389,13 +23378,13 @@
     </row>
     <row r="291" spans="1:42" ht="14.5">
       <c r="A291" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B291" s="5" t="s">
         <v>599</v>
       </c>
       <c r="C291" s="5" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>85</v>
@@ -23447,7 +23436,7 @@
     </row>
     <row r="292" spans="1:42" ht="43.5">
       <c r="A292" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B292" s="5" t="s">
         <v>603</v>
@@ -23491,7 +23480,7 @@
         <v>55</v>
       </c>
       <c r="U292" s="5" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="V292" s="5"/>
       <c r="W292" s="5"/>
@@ -23517,7 +23506,7 @@
     </row>
     <row r="293" spans="1:42" ht="14.5">
       <c r="A293" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B293" s="5" t="s">
         <v>609</v>
@@ -23561,7 +23550,7 @@
         <v>39</v>
       </c>
       <c r="U293" s="5" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="V293" s="5"/>
       <c r="W293" s="5"/>
@@ -23587,7 +23576,7 @@
     </row>
     <row r="294" spans="1:42" ht="14.5">
       <c r="A294" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B294" s="5" t="s">
         <v>614</v>
@@ -23641,13 +23630,13 @@
     </row>
     <row r="295" spans="1:42" ht="43.5">
       <c r="A295" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B295" s="5" t="s">
         <v>616</v>
       </c>
       <c r="C295" s="5" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="D295" s="5" t="s">
         <v>38</v>
@@ -23711,7 +23700,7 @@
     </row>
     <row r="296" spans="1:42" ht="29">
       <c r="A296" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B296" s="5" t="s">
         <v>621</v>
@@ -23773,13 +23762,13 @@
     </row>
     <row r="297" spans="1:42" ht="43.5">
       <c r="A297" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B297" s="5" t="s">
         <v>546</v>
       </c>
       <c r="C297" s="5" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>85</v>
@@ -23805,7 +23794,7 @@
         <v>571</v>
       </c>
       <c r="Q297" s="5" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="R297" s="5"/>
       <c r="S297" s="5"/>
@@ -23835,13 +23824,13 @@
     </row>
     <row r="298" spans="1:42" ht="14.5">
       <c r="A298" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B298" s="5" t="s">
         <v>550</v>
       </c>
       <c r="C298" s="5" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="D298" s="5" t="s">
         <v>38</v>
@@ -23867,7 +23856,7 @@
         <v>579</v>
       </c>
       <c r="Q298" s="5" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="R298" s="5"/>
       <c r="S298" s="5"/>
@@ -23897,7 +23886,7 @@
     </row>
     <row r="299" spans="1:42" ht="29">
       <c r="A299" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B299" s="5" t="s">
         <v>554</v>
@@ -23955,7 +23944,7 @@
     </row>
     <row r="300" spans="1:42" ht="43.5">
       <c r="A300" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B300" s="5" t="s">
         <v>557</v>
@@ -23987,7 +23976,7 @@
         <v>594</v>
       </c>
       <c r="Q300" s="5" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="R300" s="5"/>
       <c r="S300" s="5"/>
@@ -24017,7 +24006,7 @@
     </row>
     <row r="301" spans="1:42" ht="14.5">
       <c r="A301" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B301" s="5" t="s">
         <v>561</v>
@@ -24071,7 +24060,7 @@
     </row>
     <row r="302" spans="1:42" ht="14.5">
       <c r="A302" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B302" s="5" t="s">
         <v>563</v>
@@ -24125,7 +24114,7 @@
     </row>
     <row r="303" spans="1:42" ht="14.5">
       <c r="A303" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B303" s="5" t="s">
         <v>565</v>
@@ -24183,13 +24172,13 @@
     </row>
     <row r="304" spans="1:42" ht="29">
       <c r="A304" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B304" s="5" t="s">
         <v>568</v>
       </c>
       <c r="C304" s="5" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>85</v>
@@ -24245,7 +24234,7 @@
     </row>
     <row r="305" spans="1:42" ht="87">
       <c r="A305" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B305" s="5" t="s">
         <v>574</v>
@@ -24315,7 +24304,7 @@
     </row>
     <row r="306" spans="1:42" ht="87">
       <c r="A306" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B306" s="5" t="s">
         <v>587</v>
@@ -24367,7 +24356,7 @@
         <v>39</v>
       </c>
       <c r="AC306" s="7" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="AD306" s="5"/>
       <c r="AE306" s="5"/>
@@ -24385,7 +24374,7 @@
     </row>
     <row r="307" spans="1:42" ht="14.5">
       <c r="A307" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B307" s="5" t="s">
         <v>625</v>
@@ -24437,7 +24426,7 @@
     </row>
     <row r="308" spans="1:42" ht="14.5">
       <c r="A308" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B308" s="5" t="s">
         <v>627</v>
@@ -24489,7 +24478,7 @@
     </row>
     <row r="309" spans="1:42" ht="14.5">
       <c r="A309" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B309" s="5" t="s">
         <v>630</v>
@@ -24541,7 +24530,7 @@
     </row>
     <row r="310" spans="1:42" ht="14.5">
       <c r="A310" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B310" s="5" t="s">
         <v>633</v>
@@ -24595,7 +24584,7 @@
     </row>
     <row r="311" spans="1:42" ht="14.5">
       <c r="A311" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B311" s="5" t="s">
         <v>638</v>
@@ -24649,7 +24638,7 @@
     </row>
     <row r="312" spans="1:42" ht="14.5">
       <c r="A312" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="B312" s="5" t="s">
         <v>641</v>

</xml_diff>

<commit_message>
feat(PDG-23): onboard DILG, CFTC, GPPB and DMW risk categories
</commit_message>
<xml_diff>
--- a/data/rules/mapping.xlsx
+++ b/data/rules/mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F899D4-B510-48A0-830F-DDE2D11E34F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EB2F51-D770-4C24-AC80-8698E24D4AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3788" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3791" uniqueCount="892">
   <si>
     <t>Entity Category</t>
   </si>
@@ -2062,12 +2062,6 @@
   </si>
   <si>
     <t>"CFTC-RED-LIST"</t>
-  </si>
-  <si>
-    <t>"GPPB_BLACKLISTED_ENTITIES"</t>
-  </si>
-  <si>
-    <t>"DMW_RECRUITMENT_AGENCIES"</t>
   </si>
   <si>
     <t>"CFTC"</t>
@@ -2838,6 +2832,15 @@
   </si>
   <si>
     <t>is_valid</t>
+  </si>
+  <si>
+    <t>"GPPB-BLACKLISTED-ENTITIES"</t>
+  </si>
+  <si>
+    <t>"DMW-RECRUITMENT-AGENCIES"</t>
+  </si>
+  <si>
+    <t>"PEP (Politically Exposed Person)"</t>
   </si>
 </sst>
 </file>
@@ -3055,7 +3058,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3137,6 +3140,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3507,16 +3513,16 @@
         <v>34</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="AN1" s="9"/>
       <c r="AO1" s="9"/>
@@ -4208,8 +4214,12 @@
       <c r="AE9" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="AF9" s="9"/>
-      <c r="AG9" s="9"/>
+      <c r="AF9" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG9" s="28" t="s">
+        <v>891</v>
+      </c>
       <c r="AH9" s="8"/>
       <c r="AI9" s="8"/>
       <c r="AJ9" s="8"/>
@@ -4615,7 +4625,9 @@
       <c r="AF13" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="AG13" s="9"/>
+      <c r="AG13" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="AH13" s="8"/>
       <c r="AI13" s="8"/>
       <c r="AJ13" s="8"/>
@@ -9634,7 +9646,7 @@
       <c r="AO85" s="9"/>
       <c r="AP85" s="9"/>
     </row>
-    <row r="86" spans="1:42" ht="58">
+    <row r="86" spans="1:42" ht="72.5">
       <c r="A86" s="5" t="s">
         <v>35</v>
       </c>
@@ -12068,7 +12080,7 @@
         <v>39</v>
       </c>
       <c r="AM120" s="9" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="AN120" s="9"/>
       <c r="AO120" s="9"/>
@@ -12430,13 +12442,13 @@
         <v>55</v>
       </c>
       <c r="AK124" s="8" t="s">
-        <v>654</v>
+        <v>889</v>
       </c>
       <c r="AL124" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM124" s="8" t="s">
-        <v>655</v>
+        <v>890</v>
       </c>
       <c r="AN124" s="9"/>
       <c r="AO124" s="9"/>
@@ -12526,19 +12538,19 @@
         <v>55</v>
       </c>
       <c r="AI125" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="AJ125" s="9" t="s">
         <v>55</v>
       </c>
       <c r="AK125" s="9" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="AL125" s="9" t="s">
         <v>55</v>
       </c>
       <c r="AM125" s="9" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="AN125" s="9"/>
       <c r="AO125" s="9"/>
@@ -12570,7 +12582,7 @@
         <v>55</v>
       </c>
       <c r="I126" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="J126" s="5" t="s">
         <v>55</v>
@@ -12584,19 +12596,19 @@
         <v>55</v>
       </c>
       <c r="O126" s="11" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="P126" s="5" t="s">
         <v>55</v>
       </c>
       <c r="Q126" s="5" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="R126" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S126" s="5" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="T126" s="5"/>
       <c r="U126" s="5"/>
@@ -12606,19 +12618,19 @@
         <v>55</v>
       </c>
       <c r="Y126" s="11" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="Z126" s="5" t="s">
         <v>55</v>
       </c>
       <c r="AA126" s="11" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="AB126" s="5" t="s">
         <v>55</v>
       </c>
       <c r="AC126" s="13" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="AD126" s="5"/>
       <c r="AE126" s="5"/>
@@ -12634,13 +12646,13 @@
         <v>55</v>
       </c>
       <c r="AK126" s="18" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="AL126" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM126" s="8" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="AN126" s="9"/>
       <c r="AO126" s="9"/>
@@ -12794,7 +12806,7 @@
         <v>39</v>
       </c>
       <c r="S128" s="5" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="T128" s="5"/>
       <c r="U128" s="5"/>
@@ -12822,7 +12834,7 @@
         <v>55</v>
       </c>
       <c r="AI128" s="8" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="AJ128" s="8"/>
       <c r="AK128" s="8"/>
@@ -12840,7 +12852,7 @@
         <v>146</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D129" s="5" t="s">
         <v>85</v>
@@ -12918,7 +12930,7 @@
         <v>156</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D130" s="5" t="s">
         <v>38</v>
@@ -13016,7 +13028,7 @@
         <v>167</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D131" s="5" t="s">
         <v>38</v>
@@ -13048,7 +13060,7 @@
         <v>39</v>
       </c>
       <c r="O131" s="5" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="P131" s="5" t="s">
         <v>173</v>
@@ -13070,7 +13082,7 @@
         <v>177</v>
       </c>
       <c r="Y131" s="5" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="Z131" s="5" t="s">
         <v>39</v>
@@ -13092,19 +13104,19 @@
         <v>39</v>
       </c>
       <c r="AI131" s="8" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="AJ131" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AK131" s="8" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="AL131" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM131" s="8" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="AN131" s="9"/>
       <c r="AO131" s="9"/>
@@ -13408,7 +13420,7 @@
         <v>39</v>
       </c>
       <c r="G137" s="5" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="H137" s="5" t="s">
         <v>213</v>
@@ -13546,13 +13558,13 @@
         <v>59</v>
       </c>
       <c r="I139" s="6" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="J139" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K139" s="6" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="L139" s="5"/>
       <c r="M139" s="5"/>
@@ -13592,7 +13604,7 @@
         <v>39</v>
       </c>
       <c r="AI139" s="8" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="AJ139" s="8"/>
       <c r="AK139" s="8"/>
@@ -13780,13 +13792,13 @@
         <v>59</v>
       </c>
       <c r="I143" s="6" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="J143" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K143" s="6" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="L143" s="5"/>
       <c r="M143" s="5"/>
@@ -13841,13 +13853,13 @@
         <v>59</v>
       </c>
       <c r="I144" s="6" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="J144" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K144" s="6" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="L144" s="5"/>
       <c r="M144" s="5"/>
@@ -13857,7 +13869,7 @@
         <v>55</v>
       </c>
       <c r="Q144" s="5" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="R144" s="5" t="s">
         <v>55</v>
@@ -13877,7 +13889,7 @@
         <v>55</v>
       </c>
       <c r="AC144" s="5" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="AD144" s="5"/>
       <c r="AE144" s="5"/>
@@ -13887,7 +13899,7 @@
         <v>55</v>
       </c>
       <c r="AI144" s="8" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="AJ144" s="5"/>
       <c r="AK144" s="5"/>
@@ -13918,13 +13930,13 @@
         <v>59</v>
       </c>
       <c r="I145" s="6" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="J145" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K145" s="6" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="L145" s="5"/>
       <c r="M145" s="5"/>
@@ -13952,7 +13964,7 @@
         <v>55</v>
       </c>
       <c r="AI145" s="8" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="AJ145" s="5"/>
       <c r="AK145" s="5"/>
@@ -14023,7 +14035,7 @@
         <v>323</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="D147" s="5" t="s">
         <v>85</v>
@@ -14085,7 +14097,7 @@
         <v>329</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D148" s="5" t="s">
         <v>38</v>
@@ -14099,13 +14111,13 @@
         <v>59</v>
       </c>
       <c r="I148" s="6" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="J148" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K148" s="5" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="L148" s="5"/>
       <c r="M148" s="5"/>
@@ -14125,7 +14137,7 @@
         <v>55</v>
       </c>
       <c r="AA148" s="5" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="AB148" s="5"/>
       <c r="AC148" s="5"/>
@@ -14137,7 +14149,7 @@
         <v>55</v>
       </c>
       <c r="AI148" s="8" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="AJ148" s="5"/>
       <c r="AK148" s="5"/>
@@ -14227,13 +14239,13 @@
         <v>59</v>
       </c>
       <c r="I150" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="J150" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K150" s="5" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="L150" s="5"/>
       <c r="M150" s="5"/>
@@ -14261,7 +14273,7 @@
         <v>238</v>
       </c>
       <c r="AI150" s="19" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="AJ150" s="5"/>
       <c r="AK150" s="5"/>
@@ -14323,7 +14335,7 @@
         <v>39</v>
       </c>
       <c r="AI151" s="8" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="AJ151" s="8"/>
       <c r="AK151" s="8"/>
@@ -14341,7 +14353,7 @@
         <v>491</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="D152" s="5" t="s">
         <v>85</v>
@@ -14383,7 +14395,7 @@
         <v>149</v>
       </c>
       <c r="Y152" s="5" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="Z152" s="5" t="s">
         <v>149</v>
@@ -14407,7 +14419,7 @@
       <c r="AO152" s="9"/>
       <c r="AP152" s="9"/>
     </row>
-    <row r="153" spans="1:42" ht="58">
+    <row r="153" spans="1:42" ht="72.5">
       <c r="A153" s="5" t="s">
         <v>644</v>
       </c>
@@ -14449,7 +14461,7 @@
         <v>213</v>
       </c>
       <c r="Q153" s="5" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="R153" s="5"/>
       <c r="S153" s="5"/>
@@ -14461,7 +14473,7 @@
         <v>213</v>
       </c>
       <c r="Y153" s="5" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="Z153" s="5" t="s">
         <v>213</v>
@@ -14485,13 +14497,13 @@
         <v>39</v>
       </c>
       <c r="AK153" s="8" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="AL153" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM153" s="8" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="AN153" s="9"/>
       <c r="AO153" s="9"/>
@@ -14741,7 +14753,7 @@
         <v>39</v>
       </c>
       <c r="Y157" s="5" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="Z157" s="5" t="s">
         <v>39</v>
@@ -14763,7 +14775,7 @@
         <v>39</v>
       </c>
       <c r="AM157" s="8" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="AN157" s="9"/>
       <c r="AO157" s="9"/>
@@ -14815,7 +14827,7 @@
         <v>39</v>
       </c>
       <c r="Y158" s="5" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="Z158" s="5" t="s">
         <v>39</v>
@@ -14889,7 +14901,7 @@
         <v>39</v>
       </c>
       <c r="Y159" s="5" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="Z159" s="5" t="s">
         <v>39</v>
@@ -14909,13 +14921,13 @@
         <v>55</v>
       </c>
       <c r="AK159" s="8" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="AL159" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM159" s="8" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="AN159" s="9"/>
       <c r="AO159" s="9"/>
@@ -14971,7 +14983,7 @@
         <v>39</v>
       </c>
       <c r="Y160" s="5" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="Z160" s="5" t="s">
         <v>39</v>
@@ -15033,7 +15045,7 @@
         <v>39</v>
       </c>
       <c r="Y161" s="5" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="Z161" s="5" t="s">
         <v>39</v>
@@ -15055,7 +15067,7 @@
         <v>213</v>
       </c>
       <c r="AM161" s="27" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="AN161" s="9"/>
       <c r="AO161" s="9"/>
@@ -15069,7 +15081,7 @@
         <v>420</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="D162" s="5" t="s">
         <v>85</v>
@@ -15115,7 +15127,7 @@
         <v>149</v>
       </c>
       <c r="Y162" s="5" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="Z162" s="5"/>
       <c r="AA162" s="5"/>
@@ -15267,7 +15279,7 @@
         <v>39</v>
       </c>
       <c r="Y164" s="5" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="Z164" s="5"/>
       <c r="AA164" s="5"/>
@@ -15501,7 +15513,7 @@
         <v>213</v>
       </c>
       <c r="Y168" s="5" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="Z168" s="5"/>
       <c r="AA168" s="5"/>
@@ -15961,7 +15973,7 @@
         <v>571</v>
       </c>
       <c r="Q174" s="5" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="R174" s="5"/>
       <c r="S174" s="5"/>
@@ -16027,7 +16039,7 @@
         <v>579</v>
       </c>
       <c r="Q175" s="5" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="R175" s="5"/>
       <c r="S175" s="5"/>
@@ -16049,19 +16061,19 @@
         <v>55</v>
       </c>
       <c r="AI175" s="8" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="AJ175" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AK175" s="8" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="AL175" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM175" s="9" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="AO175" s="9"/>
       <c r="AP175" s="9"/>
@@ -16165,7 +16177,7 @@
         <v>39</v>
       </c>
       <c r="Q177" s="5" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="R177" s="5"/>
       <c r="S177" s="5"/>
@@ -16187,19 +16199,19 @@
         <v>39</v>
       </c>
       <c r="AI177" s="8" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="AJ177" s="8" t="s">
         <v>180</v>
       </c>
       <c r="AK177" s="8" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="AL177" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM177" s="9" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="AO177" s="9"/>
       <c r="AP177" s="9"/>
@@ -16368,7 +16380,7 @@
         <v>55</v>
       </c>
       <c r="AI180" s="8" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="AJ180" s="8"/>
       <c r="AK180" s="8"/>
@@ -16386,7 +16398,7 @@
         <v>349</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D181" s="5" t="s">
         <v>85</v>
@@ -16413,10 +16425,10 @@
       <c r="N181" s="5"/>
       <c r="O181" s="5"/>
       <c r="P181" s="5" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="Q181" s="5" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="R181" s="5"/>
       <c r="S181" s="5"/>
@@ -16452,7 +16464,7 @@
         <v>358</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="D182" s="5" t="s">
         <v>38</v>
@@ -16487,16 +16499,16 @@
         <v>364</v>
       </c>
       <c r="P182" s="5" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="Q182" s="5" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="R182" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S182" s="5" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="T182" s="5"/>
       <c r="U182" s="5"/>
@@ -16506,7 +16518,7 @@
         <v>579</v>
       </c>
       <c r="Y182" s="5" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="Z182" s="5" t="s">
         <v>372</v>
@@ -16530,7 +16542,7 @@
         <v>55</v>
       </c>
       <c r="AK182" s="8" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="AL182" s="8"/>
       <c r="AM182" s="8"/>
@@ -16546,7 +16558,7 @@
         <v>375</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="D183" s="5" t="s">
         <v>38</v>
@@ -16581,10 +16593,10 @@
         <v>380</v>
       </c>
       <c r="P183" s="5" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="Q183" s="5" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="R183" s="5" t="s">
         <v>39</v>
@@ -16600,7 +16612,7 @@
         <v>180</v>
       </c>
       <c r="Y183" s="5" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="Z183" s="5" t="s">
         <v>379</v>
@@ -16624,7 +16636,7 @@
         <v>39</v>
       </c>
       <c r="AK183" s="8" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="AL183" s="8"/>
       <c r="AM183" s="8"/>
@@ -16762,7 +16774,7 @@
         <v>397</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="D186" s="5" t="s">
         <v>38</v>
@@ -16824,7 +16836,7 @@
         <v>391</v>
       </c>
       <c r="C187" s="5" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>38</v>
@@ -16916,13 +16928,13 @@
         <v>579</v>
       </c>
       <c r="Q188" s="5" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="R188" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S188" s="5" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="T188" s="5"/>
       <c r="U188" s="5"/>
@@ -16944,7 +16956,7 @@
         <v>55</v>
       </c>
       <c r="AK188" s="8" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="AL188" s="8"/>
       <c r="AM188" s="8"/>
@@ -16960,7 +16972,7 @@
         <v>415</v>
       </c>
       <c r="C189" s="5" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>85</v>
@@ -16990,7 +17002,7 @@
         <v>352</v>
       </c>
       <c r="Q189" s="5" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="R189" s="5"/>
       <c r="S189" s="5"/>
@@ -17026,7 +17038,7 @@
         <v>417</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>38</v>
@@ -17040,23 +17052,23 @@
         <v>59</v>
       </c>
       <c r="I190" s="6" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="J190" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K190" s="5" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="L190" s="5"/>
       <c r="M190" s="5"/>
       <c r="N190" s="5"/>
       <c r="O190" s="5"/>
       <c r="P190" s="5" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="Q190" s="5" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="R190" s="5"/>
       <c r="S190" s="5"/>
@@ -17078,7 +17090,7 @@
         <v>55</v>
       </c>
       <c r="AI190" s="8" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="AJ190" s="8"/>
       <c r="AK190" s="8"/>
@@ -17086,7 +17098,7 @@
         <v>93</v>
       </c>
       <c r="AM190" s="27" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="AN190" s="9"/>
       <c r="AO190" s="9"/>
@@ -17100,7 +17112,7 @@
         <v>418</v>
       </c>
       <c r="C191" s="5" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>38</v>
@@ -17114,13 +17126,13 @@
         <v>59</v>
       </c>
       <c r="I191" s="6" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="J191" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K191" s="5" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="L191" s="5"/>
       <c r="M191" s="5"/>
@@ -17130,7 +17142,7 @@
         <v>39</v>
       </c>
       <c r="Q191" s="5" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="R191" s="5"/>
       <c r="S191" s="5"/>
@@ -17152,15 +17164,15 @@
         <v>39</v>
       </c>
       <c r="AI191" s="8" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="AJ191" s="8"/>
       <c r="AK191" s="8"/>
       <c r="AL191" s="26" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="AM191" s="26" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="AN191" s="9"/>
       <c r="AO191" s="9"/>
@@ -17174,7 +17186,7 @@
         <v>419</v>
       </c>
       <c r="C192" s="5" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="D192" s="5" t="s">
         <v>38</v>
@@ -17225,16 +17237,16 @@
         <v>644</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="C193" s="5" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="D193" s="5" t="s">
         <v>85</v>
       </c>
       <c r="E193" s="5" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="F193" s="5"/>
       <c r="G193" s="5"/>
@@ -17258,7 +17270,7 @@
         <v>149</v>
       </c>
       <c r="Q193" s="5" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="R193" s="5"/>
       <c r="S193" s="5"/>
@@ -17291,16 +17303,16 @@
         <v>644</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="D194" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E194" s="5" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="F194" s="5"/>
       <c r="G194" s="5"/>
@@ -17308,13 +17320,13 @@
         <v>59</v>
       </c>
       <c r="I194" s="6" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="J194" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K194" s="5" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="L194" s="5"/>
       <c r="M194" s="5"/>
@@ -17324,7 +17336,7 @@
         <v>55</v>
       </c>
       <c r="Q194" s="5" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="R194" s="5" t="s">
         <v>39</v>
@@ -17363,16 +17375,16 @@
         <v>644</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C195" s="5" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="D195" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E195" s="5" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="F195" s="5" t="s">
         <v>140</v>
@@ -17384,13 +17396,13 @@
         <v>59</v>
       </c>
       <c r="I195" s="6" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="J195" s="5" t="s">
         <v>59</v>
       </c>
       <c r="K195" s="5" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="L195" s="5"/>
       <c r="M195" s="5"/>
@@ -17420,7 +17432,7 @@
         <v>39</v>
       </c>
       <c r="AI195" s="8" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="AJ195" s="8"/>
       <c r="AK195" s="8"/>
@@ -17428,7 +17440,7 @@
         <v>39</v>
       </c>
       <c r="AM195" s="8" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="AN195" s="9"/>
       <c r="AO195" s="9"/>
@@ -17439,16 +17451,16 @@
         <v>644</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="D196" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E196" s="5" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="F196" s="5"/>
       <c r="G196" s="5"/>
@@ -17466,7 +17478,7 @@
         <v>55</v>
       </c>
       <c r="S196" s="5" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="T196" s="5"/>
       <c r="U196" s="5"/>
@@ -17500,7 +17512,7 @@
         <v>599</v>
       </c>
       <c r="C197" s="5" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="D197" s="5" t="s">
         <v>85</v>
@@ -17618,19 +17630,19 @@
         <v>55</v>
       </c>
       <c r="AI198" s="8" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="AJ198" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AK198" s="8" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="AL198" s="8" t="s">
         <v>55</v>
       </c>
       <c r="AM198" s="8" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="AN198" s="9"/>
       <c r="AO198" s="9"/>
@@ -17696,19 +17708,19 @@
         <v>39</v>
       </c>
       <c r="AI199" s="8" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="AJ199" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AK199" s="8" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="AL199" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM199" s="8" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="AN199" s="9"/>
       <c r="AO199" s="9"/>
@@ -17764,13 +17776,13 @@
         <v>39</v>
       </c>
       <c r="AK200" s="8" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="AL200" s="8" t="s">
         <v>39</v>
       </c>
       <c r="AM200" s="8" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="AN200" s="9"/>
       <c r="AO200" s="9"/>
@@ -17784,7 +17796,7 @@
         <v>616</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D201" s="5" t="s">
         <v>38</v>
@@ -17848,7 +17860,7 @@
         <v>39</v>
       </c>
       <c r="AM201" s="5" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="AN201" s="9"/>
       <c r="AO201" s="9"/>
@@ -17916,13 +17928,13 @@
         <v>213</v>
       </c>
       <c r="AK202" s="8" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="AL202" s="25" t="s">
         <v>213</v>
       </c>
       <c r="AM202" s="8" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="AN202" s="9"/>
       <c r="AO202" s="9"/>
@@ -17936,7 +17948,7 @@
         <v>568</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="D203" s="5" t="s">
         <v>85</v>
@@ -18255,10 +18267,10 @@
       <c r="AH207" s="8"/>
       <c r="AI207" s="8"/>
       <c r="AJ207" s="26" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="AK207" s="26" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="AL207" s="5"/>
       <c r="AM207" s="5"/>
@@ -18311,10 +18323,10 @@
       <c r="AH208" s="5"/>
       <c r="AI208" s="5"/>
       <c r="AJ208" s="26" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="AK208" s="26" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="AL208" s="5"/>
       <c r="AM208" s="5"/>
@@ -18370,7 +18382,7 @@
         <v>149</v>
       </c>
       <c r="AI209" s="8" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="AJ209" s="8"/>
       <c r="AK209" s="8"/>
@@ -18428,7 +18440,7 @@
         <v>39</v>
       </c>
       <c r="AI210" s="5" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="AJ210" s="5"/>
       <c r="AK210" s="5"/>
@@ -18498,7 +18510,7 @@
     </row>
     <row r="212" spans="1:42" ht="14.5">
       <c r="A212" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B212" s="5" t="s">
         <v>36</v>
@@ -18540,7 +18552,7 @@
         <v>39</v>
       </c>
       <c r="U212" s="5" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="V212" s="5"/>
       <c r="W212" s="5"/>
@@ -18570,13 +18582,13 @@
     </row>
     <row r="213" spans="1:42" ht="14.5">
       <c r="A213" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B213" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="D213" s="5" t="s">
         <v>38</v>
@@ -18604,7 +18616,7 @@
         <v>55</v>
       </c>
       <c r="Q213" s="5" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="R213" s="5"/>
       <c r="S213" s="5"/>
@@ -18612,7 +18624,7 @@
         <v>55</v>
       </c>
       <c r="U213" s="5" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="V213" s="5"/>
       <c r="W213" s="5"/>
@@ -18624,7 +18636,7 @@
         <v>55</v>
       </c>
       <c r="AC213" s="7" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="AD213" s="5"/>
       <c r="AE213" s="5"/>
@@ -18642,13 +18654,13 @@
     </row>
     <row r="214" spans="1:42" ht="14.5">
       <c r="A214" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B214" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C214" s="5" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="D214" s="5" t="s">
         <v>38</v>
@@ -18680,7 +18692,7 @@
         <v>39</v>
       </c>
       <c r="U214" s="5" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="V214" s="5"/>
       <c r="W214" s="5"/>
@@ -18710,7 +18722,7 @@
     </row>
     <row r="215" spans="1:42" ht="14.5">
       <c r="A215" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B215" s="5" t="s">
         <v>76</v>
@@ -18770,7 +18782,7 @@
     </row>
     <row r="216" spans="1:42" ht="14.5">
       <c r="A216" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B216" s="5" t="s">
         <v>83</v>
@@ -18824,7 +18836,7 @@
     </row>
     <row r="217" spans="1:42" ht="29">
       <c r="A217" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B217" s="5" t="s">
         <v>87</v>
@@ -18898,7 +18910,7 @@
     </row>
     <row r="218" spans="1:42" ht="29">
       <c r="A218" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B218" s="5" t="s">
         <v>90</v>
@@ -18988,7 +19000,7 @@
     </row>
     <row r="219" spans="1:42" ht="14.5">
       <c r="A219" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B219" s="5" t="s">
         <v>97</v>
@@ -19032,7 +19044,7 @@
         <v>55</v>
       </c>
       <c r="U219" s="5" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="V219" s="5"/>
       <c r="W219" s="5"/>
@@ -19070,7 +19082,7 @@
     </row>
     <row r="220" spans="1:42" ht="14.5">
       <c r="A220" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B220" s="5" t="s">
         <v>111</v>
@@ -19144,7 +19156,7 @@
     </row>
     <row r="221" spans="1:42" ht="58">
       <c r="A221" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B221" s="5" t="s">
         <v>122</v>
@@ -19168,7 +19180,7 @@
         <v>55</v>
       </c>
       <c r="I221" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="J221" s="5"/>
       <c r="K221" s="5"/>
@@ -19180,7 +19192,7 @@
         <v>55</v>
       </c>
       <c r="Q221" s="5" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="R221" s="5"/>
       <c r="S221" s="5"/>
@@ -19188,7 +19200,7 @@
         <v>39</v>
       </c>
       <c r="U221" s="21" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="V221" s="5"/>
       <c r="W221" s="5"/>
@@ -19200,7 +19212,7 @@
         <v>55</v>
       </c>
       <c r="AC221" s="13" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="AD221" s="5"/>
       <c r="AE221" s="5"/>
@@ -19218,7 +19230,7 @@
     </row>
     <row r="222" spans="1:42" ht="14.5">
       <c r="A222" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B222" s="5" t="s">
         <v>136</v>
@@ -19262,7 +19274,7 @@
         <v>39</v>
       </c>
       <c r="U222" s="5" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="V222" s="5"/>
       <c r="W222" s="5"/>
@@ -19292,7 +19304,7 @@
     </row>
     <row r="223" spans="1:42" ht="14.5">
       <c r="A223" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B223" s="5" t="s">
         <v>138</v>
@@ -19358,13 +19370,13 @@
     </row>
     <row r="224" spans="1:42" ht="29">
       <c r="A224" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B224" s="5" t="s">
         <v>146</v>
       </c>
       <c r="C224" s="5" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="D224" s="5" t="s">
         <v>85</v>
@@ -19424,13 +19436,13 @@
     </row>
     <row r="225" spans="1:42" ht="43.5">
       <c r="A225" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B225" s="5" t="s">
         <v>156</v>
       </c>
       <c r="C225" s="5" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="D225" s="5" t="s">
         <v>38</v>
@@ -19498,13 +19510,13 @@
     </row>
     <row r="226" spans="1:42" ht="58">
       <c r="A226" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B226" s="5" t="s">
         <v>167</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="D226" s="5" t="s">
         <v>38</v>
@@ -19542,7 +19554,7 @@
         <v>39</v>
       </c>
       <c r="U226" s="5" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="V226" s="5"/>
       <c r="W226" s="5"/>
@@ -19554,7 +19566,7 @@
         <v>39</v>
       </c>
       <c r="AC226" s="7" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="AD226" s="5"/>
       <c r="AE226" s="5"/>
@@ -19572,7 +19584,7 @@
     </row>
     <row r="227" spans="1:42" ht="14.5">
       <c r="A227" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B227" s="5" t="s">
         <v>200</v>
@@ -19624,7 +19636,7 @@
     </row>
     <row r="228" spans="1:42" ht="14.5">
       <c r="A228" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B228" s="5" t="s">
         <v>201</v>
@@ -19676,7 +19688,7 @@
     </row>
     <row r="229" spans="1:42" ht="14.5">
       <c r="A229" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B229" s="5" t="s">
         <v>202</v>
@@ -19728,7 +19740,7 @@
     </row>
     <row r="230" spans="1:42" ht="14.5">
       <c r="A230" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B230" s="5" t="s">
         <v>203</v>
@@ -19782,7 +19794,7 @@
     </row>
     <row r="231" spans="1:42" ht="14.5">
       <c r="A231" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B231" s="5" t="s">
         <v>209</v>
@@ -19838,7 +19850,7 @@
     </row>
     <row r="232" spans="1:42" ht="14.5">
       <c r="A232" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B232" s="5" t="s">
         <v>211</v>
@@ -19858,7 +19870,7 @@
         <v>59</v>
       </c>
       <c r="I232" s="6" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="J232" s="5"/>
       <c r="K232" s="5"/>
@@ -19896,13 +19908,13 @@
     </row>
     <row r="233" spans="1:42" ht="14.5">
       <c r="A233" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B233" s="5" t="s">
         <v>420</v>
       </c>
       <c r="C233" s="5" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="D233" s="5" t="s">
         <v>85</v>
@@ -19962,7 +19974,7 @@
     </row>
     <row r="234" spans="1:42" ht="43.5">
       <c r="A234" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B234" s="5" t="s">
         <v>425</v>
@@ -20032,7 +20044,7 @@
     </row>
     <row r="235" spans="1:42" ht="43.5">
       <c r="A235" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B235" s="5" t="s">
         <v>430</v>
@@ -20102,7 +20114,7 @@
     </row>
     <row r="236" spans="1:42" ht="14.5">
       <c r="A236" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B236" s="5" t="s">
         <v>437</v>
@@ -20154,7 +20166,7 @@
     </row>
     <row r="237" spans="1:42" ht="14.5">
       <c r="A237" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B237" s="5" t="s">
         <v>438</v>
@@ -20206,7 +20218,7 @@
     </row>
     <row r="238" spans="1:42" ht="14.5">
       <c r="A238" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B238" s="5" t="s">
         <v>439</v>
@@ -20258,7 +20270,7 @@
     </row>
     <row r="239" spans="1:42" ht="43.5">
       <c r="A239" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B239" s="5" t="s">
         <v>440</v>
@@ -20282,7 +20294,7 @@
         <v>59</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="J239" s="5"/>
       <c r="K239" s="5"/>
@@ -20324,13 +20336,13 @@
     </row>
     <row r="240" spans="1:42" ht="29">
       <c r="A240" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B240" s="5" t="s">
         <v>349</v>
       </c>
       <c r="C240" s="5" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D240" s="5" t="s">
         <v>85</v>
@@ -20353,10 +20365,10 @@
       <c r="N240" s="5"/>
       <c r="O240" s="5"/>
       <c r="P240" s="5" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="Q240" s="5" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="R240" s="5"/>
       <c r="S240" s="5"/>
@@ -20386,13 +20398,13 @@
     </row>
     <row r="241" spans="1:42" ht="188.5">
       <c r="A241" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B241" s="5" t="s">
         <v>358</v>
       </c>
       <c r="C241" s="5" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="D241" s="5" t="s">
         <v>38</v>
@@ -20404,7 +20416,7 @@
         <v>372</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="H241" s="5" t="s">
         <v>361</v>
@@ -20419,10 +20431,10 @@
       <c r="N241" s="5"/>
       <c r="O241" s="5"/>
       <c r="P241" s="5" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="Q241" s="5" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="R241" s="5"/>
       <c r="S241" s="5"/>
@@ -20430,7 +20442,7 @@
         <v>55</v>
       </c>
       <c r="U241" s="5" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="V241" s="5"/>
       <c r="W241" s="5"/>
@@ -20442,7 +20454,7 @@
         <v>93</v>
       </c>
       <c r="AC241" s="7" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="AD241" s="5"/>
       <c r="AE241" s="5"/>
@@ -20460,13 +20472,13 @@
     </row>
     <row r="242" spans="1:42" ht="145">
       <c r="A242" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B242" s="5" t="s">
         <v>375</v>
       </c>
       <c r="C242" s="5" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="D242" s="5" t="s">
         <v>38</v>
@@ -20478,13 +20490,13 @@
         <v>379</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="H242" s="5" t="s">
         <v>377</v>
       </c>
       <c r="I242" s="6" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="J242" s="5"/>
       <c r="K242" s="5"/>
@@ -20493,10 +20505,10 @@
       <c r="N242" s="5"/>
       <c r="O242" s="5"/>
       <c r="P242" s="5" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="Q242" s="5" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="R242" s="5"/>
       <c r="S242" s="5"/>
@@ -20504,7 +20516,7 @@
         <v>39</v>
       </c>
       <c r="U242" s="5" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="V242" s="5"/>
       <c r="W242" s="5"/>
@@ -20516,7 +20528,7 @@
         <v>180</v>
       </c>
       <c r="AC242" s="7" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="AD242" s="5"/>
       <c r="AE242" s="5"/>
@@ -20534,7 +20546,7 @@
     </row>
     <row r="243" spans="1:42" ht="29">
       <c r="A243" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B243" s="5" t="s">
         <v>390</v>
@@ -20586,13 +20598,13 @@
     </row>
     <row r="244" spans="1:42" ht="14.5">
       <c r="A244" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B244" s="5" t="s">
         <v>397</v>
       </c>
       <c r="C244" s="5" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="D244" s="5" t="s">
         <v>38</v>
@@ -20644,13 +20656,13 @@
     </row>
     <row r="245" spans="1:42" ht="14.5">
       <c r="A245" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B245" s="5" t="s">
         <v>391</v>
       </c>
       <c r="C245" s="5" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="D245" s="5" t="s">
         <v>38</v>
@@ -20702,13 +20714,13 @@
     </row>
     <row r="246" spans="1:42" ht="14.5">
       <c r="A246" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B246" s="5" t="s">
         <v>401</v>
       </c>
       <c r="C246" s="5" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="D246" s="5" t="s">
         <v>38</v>
@@ -20760,7 +20772,7 @@
     </row>
     <row r="247" spans="1:42" ht="174">
       <c r="A247" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B247" s="5" t="s">
         <v>406</v>
@@ -20789,10 +20801,10 @@
       <c r="N247" s="5"/>
       <c r="O247" s="5"/>
       <c r="P247" s="5" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="Q247" s="5" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="R247" s="5"/>
       <c r="S247" s="5"/>
@@ -20822,7 +20834,7 @@
     </row>
     <row r="248" spans="1:42" ht="14.5">
       <c r="A248" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B248" s="5" t="s">
         <v>258</v>
@@ -20856,7 +20868,7 @@
         <v>149</v>
       </c>
       <c r="Q248" s="5" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="R248" s="5"/>
       <c r="S248" s="5"/>
@@ -20886,7 +20898,7 @@
     </row>
     <row r="249" spans="1:42" ht="29">
       <c r="A249" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B249" s="5" t="s">
         <v>264</v>
@@ -20906,7 +20918,7 @@
         <v>59</v>
       </c>
       <c r="I249" s="6" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="J249" s="5"/>
       <c r="K249" s="5"/>
@@ -20918,7 +20930,7 @@
         <v>39</v>
       </c>
       <c r="Q249" s="5" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="R249" s="5"/>
       <c r="S249" s="5"/>
@@ -20948,7 +20960,7 @@
     </row>
     <row r="250" spans="1:42" ht="14.5">
       <c r="A250" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B250" s="5" t="s">
         <v>276</v>
@@ -21002,7 +21014,7 @@
     </row>
     <row r="251" spans="1:42" ht="14.5">
       <c r="A251" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B251" s="5" t="s">
         <v>278</v>
@@ -21056,7 +21068,7 @@
     </row>
     <row r="252" spans="1:42" ht="14.5">
       <c r="A252" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B252" s="5" t="s">
         <v>280</v>
@@ -21110,7 +21122,7 @@
     </row>
     <row r="253" spans="1:42" ht="14.5">
       <c r="A253" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B253" s="5" t="s">
         <v>282</v>
@@ -21130,7 +21142,7 @@
         <v>59</v>
       </c>
       <c r="I253" s="6" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="J253" s="5"/>
       <c r="K253" s="5"/>
@@ -21168,7 +21180,7 @@
     </row>
     <row r="254" spans="1:42" ht="29">
       <c r="A254" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B254" s="5" t="s">
         <v>285</v>
@@ -21188,7 +21200,7 @@
         <v>59</v>
       </c>
       <c r="I254" s="6" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="J254" s="5"/>
       <c r="K254" s="5"/>
@@ -21200,7 +21212,7 @@
         <v>55</v>
       </c>
       <c r="Q254" s="5" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="R254" s="5"/>
       <c r="S254" s="5"/>
@@ -21230,7 +21242,7 @@
     </row>
     <row r="255" spans="1:42" ht="14.5">
       <c r="A255" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B255" s="5" t="s">
         <v>293</v>
@@ -21284,7 +21296,7 @@
     </row>
     <row r="256" spans="1:42" ht="14.5">
       <c r="A256" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B256" s="5" t="s">
         <v>286</v>
@@ -21338,13 +21350,13 @@
     </row>
     <row r="257" spans="1:42" ht="29">
       <c r="A257" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B257" s="5" t="s">
         <v>323</v>
       </c>
       <c r="C257" s="5" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="D257" s="5" t="s">
         <v>85</v>
@@ -21366,7 +21378,7 @@
         <v>149</v>
       </c>
       <c r="Q257" s="5" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="R257" s="5"/>
       <c r="S257" s="5"/>
@@ -21396,13 +21408,13 @@
     </row>
     <row r="258" spans="1:42" ht="14.5">
       <c r="A258" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B258" s="5" t="s">
         <v>329</v>
       </c>
       <c r="C258" s="5" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="D258" s="5" t="s">
         <v>38</v>
@@ -21424,7 +21436,7 @@
         <v>55</v>
       </c>
       <c r="Q258" s="5" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="R258" s="5"/>
       <c r="S258" s="5"/>
@@ -21454,7 +21466,7 @@
     </row>
     <row r="259" spans="1:42" ht="14.5">
       <c r="A259" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B259" s="5" t="s">
         <v>335</v>
@@ -21508,7 +21520,7 @@
     </row>
     <row r="260" spans="1:42" ht="29">
       <c r="A260" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B260" s="5" t="s">
         <v>337</v>
@@ -21536,7 +21548,7 @@
         <v>39</v>
       </c>
       <c r="Q260" s="5" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="R260" s="5"/>
       <c r="S260" s="5"/>
@@ -21566,7 +21578,7 @@
     </row>
     <row r="261" spans="1:42" ht="14.5">
       <c r="A261" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B261" s="5" t="s">
         <v>345</v>
@@ -21620,13 +21632,13 @@
     </row>
     <row r="262" spans="1:42" ht="14.5">
       <c r="A262" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B262" s="5" t="s">
         <v>491</v>
       </c>
       <c r="C262" s="5" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="D262" s="5" t="s">
         <v>85</v>
@@ -21678,7 +21690,7 @@
     </row>
     <row r="263" spans="1:42" ht="14.5">
       <c r="A263" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B263" s="5" t="s">
         <v>498</v>
@@ -21740,7 +21752,7 @@
     </row>
     <row r="264" spans="1:42" ht="29">
       <c r="A264" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B264" s="5" t="s">
         <v>507</v>
@@ -21798,7 +21810,7 @@
     </row>
     <row r="265" spans="1:42" ht="29">
       <c r="A265" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B265" s="5" t="s">
         <v>511</v>
@@ -21856,7 +21868,7 @@
     </row>
     <row r="266" spans="1:42" ht="29">
       <c r="A266" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B266" s="5" t="s">
         <v>515</v>
@@ -21914,7 +21926,7 @@
     </row>
     <row r="267" spans="1:42" ht="29">
       <c r="A267" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B267" s="5" t="s">
         <v>519</v>
@@ -21972,7 +21984,7 @@
     </row>
     <row r="268" spans="1:42" ht="29">
       <c r="A268" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B268" s="5" t="s">
         <v>530</v>
@@ -22030,7 +22042,7 @@
     </row>
     <row r="269" spans="1:42" ht="14.5">
       <c r="A269" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B269" s="5" t="s">
         <v>524</v>
@@ -22088,7 +22100,7 @@
     </row>
     <row r="270" spans="1:42" ht="29">
       <c r="A270" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B270" s="5" t="s">
         <v>535</v>
@@ -22146,7 +22158,7 @@
     </row>
     <row r="271" spans="1:42" ht="14.5">
       <c r="A271" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B271" s="5" t="s">
         <v>541</v>
@@ -22200,19 +22212,19 @@
     </row>
     <row r="272" spans="1:42" ht="14.5">
       <c r="A272" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="C272" s="5" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="D272" s="5" t="s">
         <v>85</v>
       </c>
       <c r="E272" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F272" s="5"/>
       <c r="G272" s="5"/>
@@ -22232,7 +22244,7 @@
         <v>149</v>
       </c>
       <c r="Q272" s="5" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="R272" s="5"/>
       <c r="S272" s="5"/>
@@ -22262,19 +22274,19 @@
     </row>
     <row r="273" spans="1:42" ht="14.5">
       <c r="A273" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="C273" s="5" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="D273" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E273" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F273" s="5"/>
       <c r="G273" s="5"/>
@@ -22282,7 +22294,7 @@
         <v>59</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="J273" s="5"/>
       <c r="K273" s="5"/>
@@ -22294,7 +22306,7 @@
         <v>39</v>
       </c>
       <c r="Q273" s="5" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="R273" s="5"/>
       <c r="S273" s="5"/>
@@ -22324,19 +22336,19 @@
     </row>
     <row r="274" spans="1:42" ht="14.5">
       <c r="A274" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="C274" s="5" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="D274" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E274" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F274" s="5"/>
       <c r="G274" s="5"/>
@@ -22344,7 +22356,7 @@
         <v>59</v>
       </c>
       <c r="I274" s="6" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="J274" s="5"/>
       <c r="K274" s="5"/>
@@ -22356,7 +22368,7 @@
         <v>39</v>
       </c>
       <c r="Q274" s="5" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="R274" s="5"/>
       <c r="S274" s="5"/>
@@ -22386,19 +22398,19 @@
     </row>
     <row r="275" spans="1:42" ht="14.5">
       <c r="A275" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="C275" s="5" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="D275" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E275" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F275" s="5"/>
       <c r="G275" s="5"/>
@@ -22406,7 +22418,7 @@
         <v>59</v>
       </c>
       <c r="I275" s="6" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="J275" s="5"/>
       <c r="K275" s="5"/>
@@ -22418,7 +22430,7 @@
         <v>39</v>
       </c>
       <c r="Q275" s="5" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="R275" s="5"/>
       <c r="S275" s="5"/>
@@ -22448,19 +22460,19 @@
     </row>
     <row r="276" spans="1:42" ht="29">
       <c r="A276" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="C276" s="5" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="D276" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E276" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F276" s="5"/>
       <c r="G276" s="5"/>
@@ -22502,19 +22514,19 @@
     </row>
     <row r="277" spans="1:42" ht="14.5">
       <c r="A277" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="C277" s="5" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="D277" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E277" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F277" s="5"/>
       <c r="G277" s="5"/>
@@ -22522,7 +22534,7 @@
         <v>59</v>
       </c>
       <c r="I277" s="6" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="J277" s="5"/>
       <c r="K277" s="5"/>
@@ -22534,7 +22546,7 @@
         <v>39</v>
       </c>
       <c r="Q277" s="5" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="R277" s="5"/>
       <c r="S277" s="5"/>
@@ -22564,19 +22576,19 @@
     </row>
     <row r="278" spans="1:42" ht="14.5">
       <c r="A278" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="C278" s="5" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="D278" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E278" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F278" s="5"/>
       <c r="G278" s="5"/>
@@ -22592,7 +22604,7 @@
         <v>39</v>
       </c>
       <c r="Q278" s="5" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="R278" s="5"/>
       <c r="S278" s="5"/>
@@ -22622,17 +22634,17 @@
     </row>
     <row r="279" spans="1:42" ht="14.5">
       <c r="A279" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="C279" s="5"/>
       <c r="D279" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E279" s="5" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="F279" s="5"/>
       <c r="G279" s="5"/>
@@ -22640,7 +22652,7 @@
         <v>59</v>
       </c>
       <c r="I279" s="6" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="J279" s="5"/>
       <c r="K279" s="5"/>
@@ -22652,7 +22664,7 @@
         <v>39</v>
       </c>
       <c r="Q279" s="5" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="R279" s="5"/>
       <c r="S279" s="5"/>
@@ -22682,17 +22694,17 @@
     </row>
     <row r="280" spans="1:42" ht="14.5">
       <c r="A280" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="C280" s="5"/>
       <c r="D280" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E280" s="5" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="F280" s="5"/>
       <c r="G280" s="5"/>
@@ -22700,7 +22712,7 @@
         <v>59</v>
       </c>
       <c r="I280" s="6" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="J280" s="5"/>
       <c r="K280" s="5"/>
@@ -22738,31 +22750,31 @@
     </row>
     <row r="281" spans="1:42" ht="14.5">
       <c r="A281" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="C281" s="5" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="D281" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E281" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F281" s="5" t="s">
         <v>39</v>
       </c>
       <c r="G281" s="5" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="H281" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I281" s="6" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="J281" s="5"/>
       <c r="K281" s="5"/>
@@ -22800,19 +22812,19 @@
     </row>
     <row r="282" spans="1:42" ht="14.5">
       <c r="A282" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B282" s="5" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="C282" s="5" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="D282" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E282" s="5" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="F282" s="5" t="s">
         <v>39</v>
@@ -22858,17 +22870,17 @@
     </row>
     <row r="283" spans="1:42" ht="14.5">
       <c r="A283" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="C283" s="5"/>
       <c r="D283" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E283" s="5" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="F283" s="5"/>
       <c r="G283" s="5"/>
@@ -22886,7 +22898,7 @@
       <c r="O283" s="5"/>
       <c r="P283" s="5"/>
       <c r="Q283" s="5" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="R283" s="5"/>
       <c r="S283" s="5"/>
@@ -22916,17 +22928,17 @@
     </row>
     <row r="284" spans="1:42" ht="43.5">
       <c r="A284" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B284" s="5" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C284" s="5"/>
       <c r="D284" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E284" s="5" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="F284" s="5"/>
       <c r="G284" s="5"/>
@@ -22934,7 +22946,7 @@
         <v>59</v>
       </c>
       <c r="I284" s="6" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="J284" s="5"/>
       <c r="K284" s="5"/>
@@ -22946,7 +22958,7 @@
         <v>579</v>
       </c>
       <c r="Q284" s="5" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="R284" s="5"/>
       <c r="S284" s="5"/>
@@ -22976,17 +22988,17 @@
     </row>
     <row r="285" spans="1:42" ht="43.5">
       <c r="A285" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B285" s="5" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="C285" s="5"/>
       <c r="D285" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E285" s="5" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="F285" s="5"/>
       <c r="G285" s="5"/>
@@ -22994,7 +23006,7 @@
         <v>59</v>
       </c>
       <c r="I285" s="6" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="J285" s="5"/>
       <c r="K285" s="5"/>
@@ -23006,7 +23018,7 @@
         <v>594</v>
       </c>
       <c r="Q285" s="5" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="R285" s="5"/>
       <c r="S285" s="5"/>
@@ -23036,7 +23048,7 @@
     </row>
     <row r="286" spans="1:42" ht="14.5">
       <c r="A286" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B286" s="5" t="s">
         <v>445</v>
@@ -23098,7 +23110,7 @@
     </row>
     <row r="287" spans="1:42" ht="14.5">
       <c r="A287" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B287" s="5" t="s">
         <v>450</v>
@@ -23168,7 +23180,7 @@
     </row>
     <row r="288" spans="1:42" ht="14.5">
       <c r="A288" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B288" s="5" t="s">
         <v>453</v>
@@ -23238,7 +23250,7 @@
     </row>
     <row r="289" spans="1:42" ht="29">
       <c r="A289" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B289" s="5" t="s">
         <v>463</v>
@@ -23308,7 +23320,7 @@
     </row>
     <row r="290" spans="1:42" ht="14.5">
       <c r="A290" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B290" s="5" t="s">
         <v>472</v>
@@ -23378,13 +23390,13 @@
     </row>
     <row r="291" spans="1:42" ht="14.5">
       <c r="A291" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B291" s="5" t="s">
         <v>599</v>
       </c>
       <c r="C291" s="5" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="D291" s="5" t="s">
         <v>85</v>
@@ -23436,7 +23448,7 @@
     </row>
     <row r="292" spans="1:42" ht="43.5">
       <c r="A292" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B292" s="5" t="s">
         <v>603</v>
@@ -23480,7 +23492,7 @@
         <v>55</v>
       </c>
       <c r="U292" s="5" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="V292" s="5"/>
       <c r="W292" s="5"/>
@@ -23506,7 +23518,7 @@
     </row>
     <row r="293" spans="1:42" ht="14.5">
       <c r="A293" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B293" s="5" t="s">
         <v>609</v>
@@ -23550,7 +23562,7 @@
         <v>39</v>
       </c>
       <c r="U293" s="5" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="V293" s="5"/>
       <c r="W293" s="5"/>
@@ -23576,7 +23588,7 @@
     </row>
     <row r="294" spans="1:42" ht="14.5">
       <c r="A294" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B294" s="5" t="s">
         <v>614</v>
@@ -23630,13 +23642,13 @@
     </row>
     <row r="295" spans="1:42" ht="43.5">
       <c r="A295" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B295" s="5" t="s">
         <v>616</v>
       </c>
       <c r="C295" s="5" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D295" s="5" t="s">
         <v>38</v>
@@ -23700,7 +23712,7 @@
     </row>
     <row r="296" spans="1:42" ht="29">
       <c r="A296" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B296" s="5" t="s">
         <v>621</v>
@@ -23762,13 +23774,13 @@
     </row>
     <row r="297" spans="1:42" ht="43.5">
       <c r="A297" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B297" s="5" t="s">
         <v>546</v>
       </c>
       <c r="C297" s="5" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="D297" s="5" t="s">
         <v>85</v>
@@ -23794,7 +23806,7 @@
         <v>571</v>
       </c>
       <c r="Q297" s="5" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="R297" s="5"/>
       <c r="S297" s="5"/>
@@ -23824,13 +23836,13 @@
     </row>
     <row r="298" spans="1:42" ht="14.5">
       <c r="A298" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B298" s="5" t="s">
         <v>550</v>
       </c>
       <c r="C298" s="5" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="D298" s="5" t="s">
         <v>38</v>
@@ -23856,7 +23868,7 @@
         <v>579</v>
       </c>
       <c r="Q298" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="R298" s="5"/>
       <c r="S298" s="5"/>
@@ -23886,7 +23898,7 @@
     </row>
     <row r="299" spans="1:42" ht="29">
       <c r="A299" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B299" s="5" t="s">
         <v>554</v>
@@ -23944,7 +23956,7 @@
     </row>
     <row r="300" spans="1:42" ht="43.5">
       <c r="A300" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B300" s="5" t="s">
         <v>557</v>
@@ -23976,7 +23988,7 @@
         <v>594</v>
       </c>
       <c r="Q300" s="5" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="R300" s="5"/>
       <c r="S300" s="5"/>
@@ -24006,7 +24018,7 @@
     </row>
     <row r="301" spans="1:42" ht="14.5">
       <c r="A301" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B301" s="5" t="s">
         <v>561</v>
@@ -24060,7 +24072,7 @@
     </row>
     <row r="302" spans="1:42" ht="14.5">
       <c r="A302" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B302" s="5" t="s">
         <v>563</v>
@@ -24114,7 +24126,7 @@
     </row>
     <row r="303" spans="1:42" ht="14.5">
       <c r="A303" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B303" s="5" t="s">
         <v>565</v>
@@ -24172,13 +24184,13 @@
     </row>
     <row r="304" spans="1:42" ht="29">
       <c r="A304" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B304" s="5" t="s">
         <v>568</v>
       </c>
       <c r="C304" s="5" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="D304" s="5" t="s">
         <v>85</v>
@@ -24234,7 +24246,7 @@
     </row>
     <row r="305" spans="1:42" ht="87">
       <c r="A305" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B305" s="5" t="s">
         <v>574</v>
@@ -24304,7 +24316,7 @@
     </row>
     <row r="306" spans="1:42" ht="87">
       <c r="A306" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B306" s="5" t="s">
         <v>587</v>
@@ -24356,7 +24368,7 @@
         <v>39</v>
       </c>
       <c r="AC306" s="7" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="AD306" s="5"/>
       <c r="AE306" s="5"/>
@@ -24374,7 +24386,7 @@
     </row>
     <row r="307" spans="1:42" ht="14.5">
       <c r="A307" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B307" s="5" t="s">
         <v>625</v>
@@ -24426,7 +24438,7 @@
     </row>
     <row r="308" spans="1:42" ht="14.5">
       <c r="A308" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B308" s="5" t="s">
         <v>627</v>
@@ -24478,7 +24490,7 @@
     </row>
     <row r="309" spans="1:42" ht="14.5">
       <c r="A309" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B309" s="5" t="s">
         <v>630</v>
@@ -24530,7 +24542,7 @@
     </row>
     <row r="310" spans="1:42" ht="14.5">
       <c r="A310" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B310" s="5" t="s">
         <v>633</v>
@@ -24584,7 +24596,7 @@
     </row>
     <row r="311" spans="1:42" ht="14.5">
       <c r="A311" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B311" s="5" t="s">
         <v>638</v>
@@ -24638,7 +24650,7 @@
     </row>
     <row r="312" spans="1:42" ht="14.5">
       <c r="A312" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B312" s="5" t="s">
         <v>641</v>

</xml_diff>

<commit_message>
feat(PDG-36): onboard US State Terrorist Exclusion watchlist
</commit_message>
<xml_diff>
--- a/data/rules/mapping.xlsx
+++ b/data/rules/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7111F8-7C08-4E97-A5E6-5A6D0DFCCC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2A4E96-E3D4-4299-9FB1-4C8BDFD72404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2170" yWindow="1850" windowWidth="15680" windowHeight="9430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="New Watchlist Mapping" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4443" uniqueCount="1079">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4483" uniqueCount="1094">
   <si>
     <t>Entity Category</t>
   </si>
@@ -3439,6 +3439,51 @@
   </si>
   <si>
     <t>detail.race_ethnicity * detail.hair * detail.eyes * detail.weight * detail.height * detail.skin_tone * detail.scar_tattoo * detail.reward * detail.wanted_in * detail.warrant_case_nr</t>
+  </si>
+  <si>
+    <t>US-STATE-TERRORIST-EXCLUSION</t>
+  </si>
+  <si>
+    <t>"US-STATE-TERRORIST-EXCLUSION"</t>
+  </si>
+  <si>
+    <t>"US-STATE"</t>
+  </si>
+  <si>
+    <t>https://www.state.gov/terrorist-exclusion-list/</t>
+  </si>
+  <si>
+    <t>"Terrorist Exclusion List (TEL) - designated under USA PATRIOT ACT section 411"</t>
+  </si>
+  <si>
+    <t>list.primary_name</t>
+  </si>
+  <si>
+    <t>list.alias_blob[]</t>
+  </si>
+  <si>
+    <t>list.alias_blob.type</t>
+  </si>
+  <si>
+    <t>list.alias_blob.value</t>
+  </si>
+  <si>
+    <t>list.section</t>
+  </si>
+  <si>
+    <t>"Immigration exclusion designation (USA PATRIOT ACT section 411)"</t>
+  </si>
+  <si>
+    <t>"Designation Criteria" * "Designation Process" * "Effects of Designation" * "Tag"</t>
+  </si>
+  <si>
+    <t>path * path * path * list_expand</t>
+  </si>
+  <si>
+    <t>list.designation_criteria * list.designation_process * list.effects_of_designation * list.tags</t>
+  </si>
+  <si>
+    <t>US-STATE-TERRORIST-EXCLUSION TYPE</t>
   </si>
 </sst>
 </file>
@@ -3789,7 +3834,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -4036,6 +4081,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4259,7 +4307,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AU1030"/>
+  <dimension ref="A1:AW1030"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -4300,9 +4348,11 @@
     <col min="45" max="45" width="28.453125" customWidth="1"/>
     <col min="46" max="46" width="40.08984375" style="81" customWidth="1"/>
     <col min="47" max="47" width="34.6328125" style="84" customWidth="1"/>
+    <col min="48" max="48" width="39.1796875" style="89" customWidth="1"/>
+    <col min="49" max="49" width="34.36328125" style="89" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="14.5">
+    <row r="1" spans="1:49" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4444,8 +4494,14 @@
       <c r="AU1" s="84" t="s">
         <v>1060</v>
       </c>
-    </row>
-    <row r="2" spans="1:47" ht="29">
+      <c r="AV1" s="77" t="s">
+        <v>1093</v>
+      </c>
+      <c r="AW1" s="77" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="2" spans="1:49" ht="29">
       <c r="A2" s="10" t="s">
         <v>41</v>
       </c>
@@ -4566,7 +4622,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:47" ht="29">
+    <row r="3" spans="1:49" ht="29">
       <c r="A3" s="10" t="s">
         <v>41</v>
       </c>
@@ -4687,7 +4743,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:47" ht="58">
+    <row r="4" spans="1:49" ht="58">
       <c r="A4" s="10" t="s">
         <v>41</v>
       </c>
@@ -4785,7 +4841,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="5" spans="1:47" ht="43.5">
+    <row r="5" spans="1:49" ht="43.5">
       <c r="A5" s="10" t="s">
         <v>41</v>
       </c>
@@ -4874,7 +4930,7 @@
       <c r="AT5" s="79"/>
       <c r="AU5" s="82"/>
     </row>
-    <row r="6" spans="1:47" ht="14.5">
+    <row r="6" spans="1:49" ht="14.5">
       <c r="A6" s="10" t="s">
         <v>41</v>
       </c>
@@ -4951,7 +5007,7 @@
       <c r="AT6" s="79"/>
       <c r="AU6" s="82"/>
     </row>
-    <row r="7" spans="1:47" ht="14.5">
+    <row r="7" spans="1:49" ht="14.5">
       <c r="A7" s="10" t="s">
         <v>41</v>
       </c>
@@ -5010,7 +5066,7 @@
       <c r="AT7" s="79"/>
       <c r="AU7" s="82"/>
     </row>
-    <row r="8" spans="1:47" ht="29">
+    <row r="8" spans="1:49" ht="29">
       <c r="A8" s="10" t="s">
         <v>41</v>
       </c>
@@ -5129,7 +5185,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:47" ht="29">
+    <row r="9" spans="1:49" ht="29">
       <c r="A9" s="10" t="s">
         <v>41</v>
       </c>
@@ -5252,7 +5308,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:47" ht="14.5">
+    <row r="10" spans="1:49" ht="14.5">
       <c r="A10" s="10" t="s">
         <v>41</v>
       </c>
@@ -5375,7 +5431,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="11" spans="1:47" ht="14.5">
+    <row r="11" spans="1:49" ht="14.5">
       <c r="A11" s="10" t="s">
         <v>41</v>
       </c>
@@ -5498,7 +5554,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="12" spans="1:47" ht="38.25" customHeight="1">
+    <row r="12" spans="1:49" ht="38.25" customHeight="1">
       <c r="A12" s="10" t="s">
         <v>41</v>
       </c>
@@ -5621,7 +5677,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="13" spans="1:47" ht="29">
+    <row r="13" spans="1:49" ht="29">
       <c r="A13" s="10" t="s">
         <v>41</v>
       </c>
@@ -5740,7 +5796,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:47" ht="29">
+    <row r="14" spans="1:49" ht="29">
       <c r="A14" s="10" t="s">
         <v>41</v>
       </c>
@@ -5823,7 +5879,7 @@
       <c r="AT14" s="79"/>
       <c r="AU14" s="82"/>
     </row>
-    <row r="15" spans="1:47" ht="29">
+    <row r="15" spans="1:49" ht="29">
       <c r="A15" s="10" t="s">
         <v>41</v>
       </c>
@@ -5910,7 +5966,7 @@
       <c r="AT15" s="79"/>
       <c r="AU15" s="82"/>
     </row>
-    <row r="16" spans="1:47" ht="43.5">
+    <row r="16" spans="1:49" ht="43.5">
       <c r="A16" s="10" t="s">
         <v>41</v>
       </c>
@@ -13298,7 +13354,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="113" spans="1:47" ht="101.5">
+    <row r="113" spans="1:49" ht="101.5">
       <c r="A113" s="10" t="s">
         <v>41</v>
       </c>
@@ -13371,7 +13427,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="114" spans="1:47" ht="29">
+    <row r="114" spans="1:49" ht="29">
       <c r="A114" s="33" t="s">
         <v>41</v>
       </c>
@@ -13438,7 +13494,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="115" spans="1:47" ht="29">
+    <row r="115" spans="1:49" ht="29">
       <c r="A115" s="33" t="s">
         <v>41</v>
       </c>
@@ -13509,7 +13565,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="116" spans="1:47" ht="26">
+    <row r="116" spans="1:49" ht="26">
       <c r="A116" s="33" t="s">
         <v>41</v>
       </c>
@@ -13580,7 +13636,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="117" spans="1:47" ht="29">
+    <row r="117" spans="1:49" ht="29">
       <c r="A117" s="10" t="s">
         <v>672</v>
       </c>
@@ -13681,8 +13737,14 @@
       <c r="AP117" s="16"/>
       <c r="AQ117" s="16"/>
       <c r="AU117" s="82"/>
-    </row>
-    <row r="118" spans="1:47" ht="29">
+      <c r="AV117" s="80" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW117" s="77" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="118" spans="1:49" ht="29">
       <c r="A118" s="10" t="s">
         <v>672</v>
       </c>
@@ -13786,8 +13848,14 @@
       <c r="AS118" s="9"/>
       <c r="AT118" s="79"/>
       <c r="AU118" s="82"/>
-    </row>
-    <row r="119" spans="1:47" ht="43.5">
+      <c r="AV118" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW118" s="12" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="119" spans="1:49" ht="43.5">
       <c r="A119" s="10" t="s">
         <v>672</v>
       </c>
@@ -13876,7 +13944,7 @@
       <c r="AT119" s="62"/>
       <c r="AU119" s="83"/>
     </row>
-    <row r="120" spans="1:47" ht="14.5">
+    <row r="120" spans="1:49" ht="14.5">
       <c r="A120" s="10" t="s">
         <v>672</v>
       </c>
@@ -13961,7 +14029,7 @@
       <c r="AT120" s="79"/>
       <c r="AU120" s="82"/>
     </row>
-    <row r="121" spans="1:47" ht="14.5">
+    <row r="121" spans="1:49" ht="14.5">
       <c r="A121" s="10" t="s">
         <v>672</v>
       </c>
@@ -14020,7 +14088,7 @@
       <c r="AT121" s="79"/>
       <c r="AU121" s="82"/>
     </row>
-    <row r="122" spans="1:47" ht="29">
+    <row r="122" spans="1:49" ht="29">
       <c r="A122" s="10" t="s">
         <v>672</v>
       </c>
@@ -14126,8 +14194,14 @@
       <c r="AS122" s="9"/>
       <c r="AT122" s="79"/>
       <c r="AU122" s="82"/>
-    </row>
-    <row r="123" spans="1:47" ht="29">
+      <c r="AV122" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW122" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="123" spans="1:49" ht="29">
       <c r="A123" s="10" t="s">
         <v>672</v>
       </c>
@@ -14241,8 +14315,14 @@
       <c r="AS123" s="9"/>
       <c r="AT123" s="79"/>
       <c r="AU123" s="82"/>
-    </row>
-    <row r="124" spans="1:47" ht="14.5">
+      <c r="AV123" s="89" t="s">
+        <v>101</v>
+      </c>
+      <c r="AW123" s="89" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="124" spans="1:49" ht="14.5">
       <c r="A124" s="10" t="s">
         <v>672</v>
       </c>
@@ -14348,8 +14428,14 @@
       <c r="AS124" s="9"/>
       <c r="AT124" s="79"/>
       <c r="AU124" s="82"/>
-    </row>
-    <row r="125" spans="1:47" ht="14.5">
+      <c r="AV124" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW124" s="89" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="125" spans="1:49" ht="14.5">
       <c r="A125" s="10" t="s">
         <v>672</v>
       </c>
@@ -14455,8 +14541,14 @@
       <c r="AS125" s="9"/>
       <c r="AT125" s="79"/>
       <c r="AU125" s="82"/>
-    </row>
-    <row r="126" spans="1:47" ht="130.5">
+      <c r="AV125" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW125" s="89" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="126" spans="1:49" ht="130.5">
       <c r="A126" s="10" t="s">
         <v>672</v>
       </c>
@@ -14562,8 +14654,14 @@
       <c r="AS126" s="9"/>
       <c r="AT126" s="79"/>
       <c r="AU126" s="82"/>
-    </row>
-    <row r="127" spans="1:47" ht="29">
+      <c r="AV126" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW126" s="78" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="127" spans="1:49" ht="29">
       <c r="A127" s="10" t="s">
         <v>672</v>
       </c>
@@ -14669,8 +14767,14 @@
       <c r="AS127" s="9"/>
       <c r="AT127" s="79"/>
       <c r="AU127" s="82"/>
-    </row>
-    <row r="128" spans="1:47" ht="29">
+      <c r="AV127" s="80" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW127" s="77" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="128" spans="1:49" ht="38.5">
       <c r="A128" s="10" t="s">
         <v>672</v>
       </c>
@@ -14758,8 +14862,14 @@
       <c r="AS128" s="9"/>
       <c r="AT128" s="79"/>
       <c r="AU128" s="82"/>
-    </row>
-    <row r="129" spans="1:47" ht="29">
+      <c r="AV128" s="89" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW128" s="90" t="s">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="129" spans="1:49" ht="29">
       <c r="A129" s="10" t="s">
         <v>672</v>
       </c>
@@ -14842,7 +14952,7 @@
       <c r="AT129" s="79"/>
       <c r="AU129" s="82"/>
     </row>
-    <row r="130" spans="1:47" ht="43.5">
+    <row r="130" spans="1:49" ht="43.5">
       <c r="A130" s="10" t="s">
         <v>672</v>
       </c>
@@ -14944,8 +15054,14 @@
       <c r="AS130" s="9"/>
       <c r="AT130" s="79"/>
       <c r="AU130" s="82"/>
-    </row>
-    <row r="131" spans="1:47" ht="58">
+      <c r="AV130" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW130" s="15" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="131" spans="1:49" ht="58">
       <c r="A131" s="10" t="s">
         <v>672</v>
       </c>
@@ -15051,8 +15167,14 @@
       <c r="AS131" s="9"/>
       <c r="AT131" s="79"/>
       <c r="AU131" s="82"/>
-    </row>
-    <row r="132" spans="1:47" ht="29">
+      <c r="AV131" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW131" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="132" spans="1:49" ht="29">
       <c r="A132" s="10" t="s">
         <v>672</v>
       </c>
@@ -15109,7 +15231,7 @@
       <c r="AT132" s="79"/>
       <c r="AU132" s="82"/>
     </row>
-    <row r="133" spans="1:47" ht="14.5">
+    <row r="133" spans="1:49" ht="14.5">
       <c r="A133" s="10" t="s">
         <v>672</v>
       </c>
@@ -15166,7 +15288,7 @@
       <c r="AT133" s="79"/>
       <c r="AU133" s="82"/>
     </row>
-    <row r="134" spans="1:47" ht="14.5">
+    <row r="134" spans="1:49" ht="14.5">
       <c r="A134" s="10" t="s">
         <v>672</v>
       </c>
@@ -15223,7 +15345,7 @@
       <c r="AT134" s="79"/>
       <c r="AU134" s="82"/>
     </row>
-    <row r="135" spans="1:47" ht="29">
+    <row r="135" spans="1:49" ht="29">
       <c r="A135" s="10" t="s">
         <v>672</v>
       </c>
@@ -15290,7 +15412,7 @@
       <c r="AT135" s="79"/>
       <c r="AU135" s="82"/>
     </row>
-    <row r="136" spans="1:47" ht="43.5">
+    <row r="136" spans="1:49" ht="43.5">
       <c r="A136" s="10" t="s">
         <v>672</v>
       </c>
@@ -15355,7 +15477,7 @@
       <c r="AT136" s="62"/>
       <c r="AU136" s="83"/>
     </row>
-    <row r="137" spans="1:47" ht="43.5">
+    <row r="137" spans="1:49" ht="43.5">
       <c r="A137" s="10" t="s">
         <v>672</v>
       </c>
@@ -15430,7 +15552,7 @@
       <c r="AT137" s="79"/>
       <c r="AU137" s="82"/>
     </row>
-    <row r="138" spans="1:47" ht="14.5">
+    <row r="138" spans="1:49" ht="14.5">
       <c r="A138" s="10" t="s">
         <v>672</v>
       </c>
@@ -15501,7 +15623,7 @@
       <c r="AT138" s="79"/>
       <c r="AU138" s="82"/>
     </row>
-    <row r="139" spans="1:47" ht="116">
+    <row r="139" spans="1:49" ht="116">
       <c r="A139" s="10" t="s">
         <v>672</v>
       </c>
@@ -15583,7 +15705,7 @@
       <c r="AT139" s="79"/>
       <c r="AU139" s="82"/>
     </row>
-    <row r="140" spans="1:47" ht="14.5">
+    <row r="140" spans="1:49" ht="14.5">
       <c r="A140" s="10" t="s">
         <v>672</v>
       </c>
@@ -15641,7 +15763,7 @@
       <c r="AT140" s="79"/>
       <c r="AU140" s="82"/>
     </row>
-    <row r="141" spans="1:47" ht="14.5">
+    <row r="141" spans="1:49" ht="14.5">
       <c r="A141" s="10" t="s">
         <v>672</v>
       </c>
@@ -15699,7 +15821,7 @@
       <c r="AT141" s="79"/>
       <c r="AU141" s="82"/>
     </row>
-    <row r="142" spans="1:47" ht="14.5">
+    <row r="142" spans="1:49" ht="14.5">
       <c r="A142" s="10" t="s">
         <v>672</v>
       </c>
@@ -15757,7 +15879,7 @@
       <c r="AT142" s="79"/>
       <c r="AU142" s="82"/>
     </row>
-    <row r="143" spans="1:47" ht="72.5">
+    <row r="143" spans="1:49" ht="72.5">
       <c r="A143" s="10" t="s">
         <v>672</v>
       </c>
@@ -15823,7 +15945,7 @@
       <c r="AT143" s="79"/>
       <c r="AU143" s="82"/>
     </row>
-    <row r="144" spans="1:47" ht="130.5">
+    <row r="144" spans="1:49" ht="130.5">
       <c r="A144" s="10" t="s">
         <v>672</v>
       </c>
@@ -17084,7 +17206,7 @@
       <c r="AT160" s="79"/>
       <c r="AU160" s="82"/>
     </row>
-    <row r="161" spans="1:47" ht="14.5">
+    <row r="161" spans="1:49" ht="14.5">
       <c r="A161" s="10" t="s">
         <v>672</v>
       </c>
@@ -17155,7 +17277,7 @@
       <c r="AT161" s="79"/>
       <c r="AU161" s="82"/>
     </row>
-    <row r="162" spans="1:47" ht="14.5">
+    <row r="162" spans="1:49" ht="14.5">
       <c r="A162" s="10" t="s">
         <v>672</v>
       </c>
@@ -17233,8 +17355,14 @@
       <c r="AS162" s="9"/>
       <c r="AT162" s="79"/>
       <c r="AU162" s="82"/>
-    </row>
-    <row r="163" spans="1:47" ht="43.5">
+      <c r="AV162" s="77" t="s">
+        <v>163</v>
+      </c>
+      <c r="AW162" s="77" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="163" spans="1:49" ht="43.5">
       <c r="A163" s="10" t="s">
         <v>672</v>
       </c>
@@ -17316,8 +17444,14 @@
       <c r="AS163" s="9"/>
       <c r="AT163" s="79"/>
       <c r="AU163" s="82"/>
-    </row>
-    <row r="164" spans="1:47" ht="58">
+      <c r="AV163" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW163" s="77" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="164" spans="1:49" ht="58">
       <c r="A164" s="10" t="s">
         <v>672</v>
       </c>
@@ -17399,8 +17533,14 @@
       <c r="AS164" s="9"/>
       <c r="AT164" s="79"/>
       <c r="AU164" s="82"/>
-    </row>
-    <row r="165" spans="1:47" ht="14.5">
+      <c r="AV164" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW164" s="89" t="s">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="165" spans="1:49" ht="14.5">
       <c r="A165" s="10" t="s">
         <v>672</v>
       </c>
@@ -17457,7 +17597,7 @@
       <c r="AT165" s="79"/>
       <c r="AU165" s="82"/>
     </row>
-    <row r="166" spans="1:47" ht="14.5">
+    <row r="166" spans="1:49" ht="14.5">
       <c r="A166" s="10" t="s">
         <v>672</v>
       </c>
@@ -17514,7 +17654,7 @@
       <c r="AT166" s="79"/>
       <c r="AU166" s="82"/>
     </row>
-    <row r="167" spans="1:47" ht="14.5">
+    <row r="167" spans="1:49" ht="14.5">
       <c r="A167" s="10" t="s">
         <v>672</v>
       </c>
@@ -17571,7 +17711,7 @@
       <c r="AT167" s="79"/>
       <c r="AU167" s="82"/>
     </row>
-    <row r="168" spans="1:47" ht="43.5">
+    <row r="168" spans="1:49" ht="43.5">
       <c r="A168" s="10" t="s">
         <v>672</v>
       </c>
@@ -17650,7 +17790,7 @@
       <c r="AT168" s="79"/>
       <c r="AU168" s="82"/>
     </row>
-    <row r="169" spans="1:47" ht="29">
+    <row r="169" spans="1:49" ht="29">
       <c r="A169" s="10" t="s">
         <v>672</v>
       </c>
@@ -17721,7 +17861,7 @@
       <c r="AT169" s="79"/>
       <c r="AU169" s="82"/>
     </row>
-    <row r="170" spans="1:47" ht="14.5">
+    <row r="170" spans="1:49" ht="14.5">
       <c r="A170" s="10" t="s">
         <v>672</v>
       </c>
@@ -17812,7 +17952,7 @@
       <c r="AT170" s="79"/>
       <c r="AU170" s="82"/>
     </row>
-    <row r="171" spans="1:47" ht="14.5">
+    <row r="171" spans="1:49" ht="14.5">
       <c r="A171" s="10" t="s">
         <v>672</v>
       </c>
@@ -17903,7 +18043,7 @@
       <c r="AT171" s="79"/>
       <c r="AU171" s="82"/>
     </row>
-    <row r="172" spans="1:47" ht="29">
+    <row r="172" spans="1:49" ht="29">
       <c r="A172" s="10" t="s">
         <v>672</v>
       </c>
@@ -17994,7 +18134,7 @@
       <c r="AT172" s="79"/>
       <c r="AU172" s="82"/>
     </row>
-    <row r="173" spans="1:47" ht="29">
+    <row r="173" spans="1:49" ht="29">
       <c r="A173" s="10" t="s">
         <v>672</v>
       </c>
@@ -18077,7 +18217,7 @@
       <c r="AT173" s="79"/>
       <c r="AU173" s="82"/>
     </row>
-    <row r="174" spans="1:47" ht="29">
+    <row r="174" spans="1:49" ht="29">
       <c r="A174" s="10" t="s">
         <v>672</v>
       </c>
@@ -18148,7 +18288,7 @@
       <c r="AT174" s="79"/>
       <c r="AU174" s="82"/>
     </row>
-    <row r="175" spans="1:47" ht="29">
+    <row r="175" spans="1:49" ht="29">
       <c r="A175" s="10" t="s">
         <v>672</v>
       </c>
@@ -18230,7 +18370,7 @@
       <c r="AT175" s="79"/>
       <c r="AU175" s="82"/>
     </row>
-    <row r="176" spans="1:47" ht="29">
+    <row r="176" spans="1:49" ht="29">
       <c r="A176" s="10" t="s">
         <v>672</v>
       </c>
@@ -19469,7 +19609,7 @@
       <c r="AT192" s="79"/>
       <c r="AU192" s="82"/>
     </row>
-    <row r="193" spans="1:47" ht="14.5">
+    <row r="193" spans="1:49" ht="14.5">
       <c r="A193" s="10" t="s">
         <v>672</v>
       </c>
@@ -19540,7 +19680,7 @@
       <c r="AT193" s="79"/>
       <c r="AU193" s="82"/>
     </row>
-    <row r="194" spans="1:47" ht="43.5">
+    <row r="194" spans="1:49" ht="43.5">
       <c r="A194" s="10" t="s">
         <v>672</v>
       </c>
@@ -19617,7 +19757,7 @@
       <c r="AT194" s="79"/>
       <c r="AU194" s="82"/>
     </row>
-    <row r="195" spans="1:47" ht="43.5">
+    <row r="195" spans="1:49" ht="43.5">
       <c r="A195" s="10" t="s">
         <v>672</v>
       </c>
@@ -19698,7 +19838,7 @@
       <c r="AT195" s="79"/>
       <c r="AU195" s="82"/>
     </row>
-    <row r="196" spans="1:47" ht="14.5">
+    <row r="196" spans="1:49" ht="14.5">
       <c r="A196" s="10" t="s">
         <v>672</v>
       </c>
@@ -19761,7 +19901,7 @@
       <c r="AT196" s="79"/>
       <c r="AU196" s="82"/>
     </row>
-    <row r="197" spans="1:47" ht="43.5">
+    <row r="197" spans="1:49" ht="43.5">
       <c r="A197" s="10" t="s">
         <v>672</v>
       </c>
@@ -19828,7 +19968,7 @@
       <c r="AT197" s="79"/>
       <c r="AU197" s="82"/>
     </row>
-    <row r="198" spans="1:47" ht="130.5">
+    <row r="198" spans="1:49" ht="145">
       <c r="A198" s="10" t="s">
         <v>672</v>
       </c>
@@ -19914,8 +20054,14 @@
       <c r="AS198" s="9"/>
       <c r="AT198" s="79"/>
       <c r="AU198" s="82"/>
-    </row>
-    <row r="199" spans="1:47" ht="43.5">
+      <c r="AV198" s="77" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW198" s="69" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="199" spans="1:49" ht="43.5">
       <c r="A199" s="10" t="s">
         <v>672</v>
       </c>
@@ -19997,8 +20143,9 @@
       <c r="AS199" s="9"/>
       <c r="AT199" s="79"/>
       <c r="AU199" s="82"/>
-    </row>
-    <row r="200" spans="1:47" ht="14.5">
+      <c r="AW199" s="69"/>
+    </row>
+    <row r="200" spans="1:49" ht="14.5">
       <c r="A200" s="10" t="s">
         <v>672</v>
       </c>
@@ -20065,7 +20212,7 @@
       <c r="AT200" s="79"/>
       <c r="AU200" s="82"/>
     </row>
-    <row r="201" spans="1:47" ht="43.5">
+    <row r="201" spans="1:49" ht="43.5">
       <c r="A201" s="10" t="s">
         <v>672</v>
       </c>
@@ -20147,8 +20294,14 @@
       <c r="AS201" s="9"/>
       <c r="AT201" s="79"/>
       <c r="AU201" s="82"/>
-    </row>
-    <row r="202" spans="1:47" ht="130.5">
+      <c r="AV201" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW201" s="69" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="202" spans="1:49" ht="130.5">
       <c r="A202" s="10" t="s">
         <v>672</v>
       </c>
@@ -20226,8 +20379,14 @@
       <c r="AS202" s="9"/>
       <c r="AT202" s="79"/>
       <c r="AU202" s="82"/>
-    </row>
-    <row r="203" spans="1:47" ht="29">
+      <c r="AV202" s="77" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW202" s="77" t="s">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="203" spans="1:49" ht="29">
       <c r="A203" s="10" t="s">
         <v>672</v>
       </c>
@@ -20298,7 +20457,7 @@
       <c r="AT203" s="79"/>
       <c r="AU203" s="82"/>
     </row>
-    <row r="204" spans="1:47" ht="377">
+    <row r="204" spans="1:49" ht="377">
       <c r="A204" s="10" t="s">
         <v>672</v>
       </c>
@@ -20385,7 +20544,7 @@
       <c r="AT204" s="79"/>
       <c r="AU204" s="82"/>
     </row>
-    <row r="205" spans="1:47" ht="391.5">
+    <row r="205" spans="1:49" ht="391.5">
       <c r="A205" s="10" t="s">
         <v>672</v>
       </c>
@@ -20472,7 +20631,7 @@
       <c r="AT205" s="79"/>
       <c r="AU205" s="82"/>
     </row>
-    <row r="206" spans="1:47" ht="14.5">
+    <row r="206" spans="1:49" ht="14.5">
       <c r="A206" s="10" t="s">
         <v>672</v>
       </c>
@@ -20529,7 +20688,7 @@
       <c r="AT206" s="79"/>
       <c r="AU206" s="82"/>
     </row>
-    <row r="207" spans="1:47" ht="29">
+    <row r="207" spans="1:49" ht="38.5">
       <c r="A207" s="10" t="s">
         <v>672</v>
       </c>
@@ -20589,8 +20748,14 @@
       <c r="AS207" s="9"/>
       <c r="AT207" s="79"/>
       <c r="AU207" s="82"/>
-    </row>
-    <row r="208" spans="1:47" ht="29">
+      <c r="AV207" s="69" t="s">
+        <v>807</v>
+      </c>
+      <c r="AW207" s="89" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="208" spans="1:49" ht="38.5">
       <c r="A208" s="10" t="s">
         <v>672</v>
       </c>
@@ -20650,6 +20815,12 @@
       <c r="AS208" s="37"/>
       <c r="AT208" s="62"/>
       <c r="AU208" s="83"/>
+      <c r="AV208" s="69" t="s">
+        <v>1091</v>
+      </c>
+      <c r="AW208" s="89" t="s">
+        <v>1092</v>
+      </c>
     </row>
     <row r="209" spans="1:47" ht="14.5">
       <c r="A209" s="33" t="s">
@@ -63653,8 +63824,9 @@
     <hyperlink ref="AC221" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="AS12" r:id="rId16" xr:uid="{119AA4A3-C354-4217-9961-39DD8D22FB3D}"/>
     <hyperlink ref="AU12" r:id="rId17" xr:uid="{5089569D-E038-4B81-AB71-AFF709AA618E}"/>
+    <hyperlink ref="AW126" r:id="rId18" xr:uid="{270161FA-D3AF-428D-897A-B60A71D0B1EB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId18"/>
+  <pageSetup orientation="portrait" r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>